<commit_message>
Unit bugfix related to weapon assignment
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Factions" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Biomes" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Combat" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Weapons" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2077,6 +2078,274 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Weapon ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Damage Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Attacks Per Second</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Windup</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Hit Mode</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Projectile Key</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Animation Key</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Target Filters</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Stat Scaling</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>weapon_fists</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fists</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unarmed strikes.</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Blunt</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>attack_fists</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Enemies</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>weapon_wolf_bite</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wolf Bite</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Natural wolf bite attack.</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>attack_bite</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>weapon_claws</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Claws</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Natural claw swipe.</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>attack_claws</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Unit facing direction of travel
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9615" yWindow="15" windowWidth="28785" windowHeight="15570" tabRatio="600" firstSheet="3" activeTab="13" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9615" yWindow="15" windowWidth="28785" windowHeight="15570" tabRatio="600" firstSheet="3" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Unit Import Schema" sheetId="1" state="visible" r:id="rId1"/>
@@ -133,10 +133,15 @@
       <sz val="12"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
@@ -244,12 +249,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -389,16 +394,16 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -906,12 +911,12 @@
   <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" style="38" min="1" max="1"/>
-    <col width="22" customWidth="1" style="38" min="2" max="3"/>
-    <col width="48" customWidth="1" style="38" min="4" max="4"/>
+    <col width="18" customWidth="1" style="41" min="1" max="1"/>
+    <col width="22" customWidth="1" style="41" min="2" max="3"/>
+    <col width="48" customWidth="1" style="41" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="38">
+    <row r="1" ht="15.75" customHeight="1" s="41">
       <c r="A1" s="35" t="inlineStr">
         <is>
           <t>Column</t>
@@ -1297,7 +1302,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="37" t="inlineStr">
+      <c r="A22" s="40" t="inlineStr">
         <is>
           <t>Importer: src/data_import/unit/schema.rs + excel.rs. Dev catalog loads this sheet at startup (feature=dev). Starter catalog (wolf/bandit/deer) is fallback only. Total Stats / Power Rating / Tier are written as plain values so calamine can read them (Excel formulas are not re-evaluated on import).</t>
         </is>
@@ -1808,20 +1813,20 @@
   <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34.85546875" bestFit="1" customWidth="1" style="38" min="1" max="1"/>
-    <col width="32.7109375" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="13.7109375" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
-    <col width="6" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
+    <col width="34.85546875" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
+    <col width="32.7109375" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="13.7109375" bestFit="1" customWidth="1" style="41" min="4" max="4"/>
+    <col width="6" bestFit="1" customWidth="1" style="41" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="38">
+    <row r="1" ht="21" customHeight="1" s="41">
       <c r="A1" s="25" t="inlineStr">
         <is>
           <t>CHASMA COMBAT SYSTEM</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" s="38">
+    <row r="3" ht="15.75" customHeight="1" s="41">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>DAMAGE CALCULATION</t>
@@ -1912,7 +1917,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1" s="38">
+    <row r="12" ht="15.75" customHeight="1" s="41">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>DEFENSE CALCULATION</t>
@@ -1991,7 +1996,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" s="38">
+    <row r="20" ht="15.75" customHeight="1" s="41">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>COMBAT EXAMPLE</t>
@@ -2116,23 +2121,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16.85546875" bestFit="1" customWidth="1" style="38" min="1" max="1"/>
-    <col width="8.7109375" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="22.42578125" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
-    <col width="8.28515625" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
-    <col width="12.7109375" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
-    <col width="6.42578125" bestFit="1" customWidth="1" style="38" min="6" max="6"/>
-    <col width="17.85546875" bestFit="1" customWidth="1" style="38" min="7" max="7"/>
-    <col width="7.85546875" bestFit="1" customWidth="1" style="38" min="8" max="8"/>
-    <col width="8.7109375" bestFit="1" customWidth="1" style="38" min="9" max="10"/>
-    <col width="12.7109375" bestFit="1" customWidth="1" style="38" min="11" max="11"/>
-    <col width="13.7109375" bestFit="1" customWidth="1" style="38" min="12" max="12"/>
-    <col width="16.28515625" bestFit="1" customWidth="1" style="38" min="13" max="13"/>
-    <col width="11.140625" bestFit="1" customWidth="1" style="38" min="14" max="14"/>
-    <col width="8.140625" bestFit="1" customWidth="1" style="38" min="15" max="15"/>
+    <col width="16.85546875" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
+    <col width="8.7109375" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="22.42578125" bestFit="1" customWidth="1" style="41" min="3" max="3"/>
+    <col width="8.28515625" bestFit="1" customWidth="1" style="41" min="4" max="4"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" style="41" min="5" max="5"/>
+    <col width="6.42578125" bestFit="1" customWidth="1" style="41" min="6" max="6"/>
+    <col width="17.85546875" bestFit="1" customWidth="1" style="41" min="7" max="7"/>
+    <col width="7.85546875" bestFit="1" customWidth="1" style="41" min="8" max="8"/>
+    <col width="8.7109375" bestFit="1" customWidth="1" style="41" min="9" max="10"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" style="41" min="11" max="11"/>
+    <col width="13.7109375" bestFit="1" customWidth="1" style="41" min="12" max="12"/>
+    <col width="16.28515625" bestFit="1" customWidth="1" style="41" min="13" max="13"/>
+    <col width="11.140625" bestFit="1" customWidth="1" style="41" min="14" max="14"/>
+    <col width="8.140625" bestFit="1" customWidth="1" style="41" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2378,6 +2383,63 @@
         </is>
       </c>
       <c r="O4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>weapon_cavecrawler_claws</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cavecrawler Claws</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Natural claw attack.</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>ClawAttackRight</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2394,7 +2456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2428,6 +2490,41 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Death Animation</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Hit Reaction Animation</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Upper Body Split Bone</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Turn Left Animation</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Turn Right Animation</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Turn Left Duration</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Turn Right Duration</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2517,6 +2614,59 @@
         <is>
           <t>Y</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cavecrawler</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>GetHit1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CrawlLeft</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>CrawlRight</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2533,10 +2683,10 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.85546875" bestFit="1" customWidth="1" style="38" min="1" max="1"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="29.7109375" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
-    <col width="8.140625" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
+    <col width="10.85546875" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="29.7109375" bestFit="1" customWidth="1" style="41" min="3" max="3"/>
+    <col width="8.140625" bestFit="1" customWidth="1" style="41" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2663,25 +2813,25 @@
   <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.28515625" bestFit="1" customWidth="1" style="38" min="1" max="1"/>
-    <col width="12.85546875" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
-    <col width="26.85546875" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
-    <col width="35.7109375" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
-    <col width="15.85546875" bestFit="1" customWidth="1" style="38" min="6" max="6"/>
-    <col width="6.7109375" bestFit="1" customWidth="1" style="38" min="7" max="7"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" style="38" min="8" max="8"/>
-    <col width="13.5703125" bestFit="1" customWidth="1" style="38" min="9" max="9"/>
-    <col width="14.7109375" bestFit="1" customWidth="1" style="38" min="10" max="11"/>
-    <col width="15.7109375" bestFit="1" customWidth="1" style="38" min="12" max="12"/>
-    <col width="9.85546875" bestFit="1" customWidth="1" style="38" min="13" max="13"/>
-    <col width="18.7109375" bestFit="1" customWidth="1" style="38" min="14" max="14"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="38" min="15" max="15"/>
-    <col width="16.42578125" bestFit="1" customWidth="1" style="38" min="16" max="16"/>
-    <col width="16.85546875" bestFit="1" customWidth="1" style="38" min="17" max="17"/>
-    <col width="13.140625" bestFit="1" customWidth="1" style="38" min="18" max="18"/>
-    <col width="8.140625" bestFit="1" customWidth="1" style="38" min="19" max="19"/>
-    <col width="17.7109375" bestFit="1" customWidth="1" style="38" min="20" max="20"/>
+    <col width="13.28515625" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
+    <col width="12.85546875" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="41" min="3" max="3"/>
+    <col width="26.85546875" bestFit="1" customWidth="1" style="41" min="4" max="4"/>
+    <col width="35.7109375" bestFit="1" customWidth="1" style="41" min="5" max="5"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" style="41" min="6" max="6"/>
+    <col width="6.7109375" bestFit="1" customWidth="1" style="41" min="7" max="7"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="41" min="8" max="8"/>
+    <col width="13.5703125" bestFit="1" customWidth="1" style="41" min="9" max="9"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" style="41" min="10" max="11"/>
+    <col width="15.7109375" bestFit="1" customWidth="1" style="41" min="12" max="12"/>
+    <col width="9.85546875" bestFit="1" customWidth="1" style="41" min="13" max="13"/>
+    <col width="18.7109375" bestFit="1" customWidth="1" style="41" min="14" max="14"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="41" min="15" max="15"/>
+    <col width="16.42578125" bestFit="1" customWidth="1" style="41" min="16" max="16"/>
+    <col width="16.85546875" bestFit="1" customWidth="1" style="41" min="17" max="17"/>
+    <col width="13.140625" bestFit="1" customWidth="1" style="41" min="18" max="18"/>
+    <col width="8.140625" bestFit="1" customWidth="1" style="41" min="19" max="19"/>
+    <col width="17.7109375" bestFit="1" customWidth="1" style="41" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3048,122 +3198,122 @@
   <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="38" min="1" max="1"/>
-    <col width="22" customWidth="1" style="38" min="2" max="2"/>
-    <col width="16" customWidth="1" style="38" min="3" max="3"/>
-    <col width="12" customWidth="1" style="38" min="4" max="4"/>
-    <col width="42" customWidth="1" style="38" min="5" max="5"/>
-    <col width="36" customWidth="1" style="38" min="6" max="6"/>
-    <col width="24" customWidth="1" style="38" min="7" max="7"/>
-    <col width="34" customWidth="1" style="38" min="8" max="8"/>
-    <col width="36" customWidth="1" style="38" min="9" max="9"/>
+    <col width="14" customWidth="1" style="41" min="1" max="1"/>
+    <col width="22" customWidth="1" style="41" min="2" max="2"/>
+    <col width="16" customWidth="1" style="41" min="3" max="3"/>
+    <col width="12" customWidth="1" style="41" min="4" max="4"/>
+    <col width="42" customWidth="1" style="41" min="5" max="5"/>
+    <col width="36" customWidth="1" style="41" min="6" max="6"/>
+    <col width="24" customWidth="1" style="41" min="7" max="7"/>
+    <col width="34" customWidth="1" style="41" min="8" max="8"/>
+    <col width="36" customWidth="1" style="41" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="40" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1" s="41">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>HOTKEY REGISTRY — Chasma</t>
         </is>
       </c>
-      <c r="B1" s="41" t="inlineStr"/>
-      <c r="C1" s="41" t="inlineStr"/>
-      <c r="D1" s="41" t="inlineStr"/>
-      <c r="E1" s="41" t="inlineStr"/>
-      <c r="F1" s="41" t="inlineStr"/>
-      <c r="G1" s="41" t="inlineStr"/>
-      <c r="H1" s="41" t="inlineStr"/>
-      <c r="I1" s="41" t="inlineStr"/>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
+      <c r="E1" s="38" t="n"/>
+      <c r="F1" s="38" t="n"/>
+      <c r="G1" s="38" t="n"/>
+      <c r="H1" s="38" t="n"/>
+      <c r="I1" s="38" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="41" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>Maintenance: update this sheet whenever keyboard bindings change in src/.</t>
         </is>
       </c>
-      <c r="B2" s="41" t="inlineStr"/>
-      <c r="C2" s="41" t="inlineStr"/>
-      <c r="D2" s="41" t="inlineStr"/>
-      <c r="E2" s="41" t="inlineStr">
+      <c r="B2" s="38" t="n"/>
+      <c r="C2" s="38" t="n"/>
+      <c r="D2" s="38" t="n"/>
+      <c r="E2" s="38" t="inlineStr">
         <is>
           <t>Regenerate: python tools/update_hotkeys_sheet.py</t>
         </is>
       </c>
-      <c r="F2" s="41" t="inlineStr">
+      <c r="F2" s="38" t="inlineStr">
         <is>
           <t>Audit code: rg 'KeyCode::' src/</t>
         </is>
       </c>
-      <c r="G2" s="41" t="inlineStr">
+      <c r="G2" s="38" t="inlineStr">
         <is>
           <t>Also update docs/dev-mode.md if player-facing</t>
         </is>
       </c>
-      <c r="H2" s="41" t="inlineStr"/>
-      <c r="I2" s="41" t="inlineStr">
+      <c r="H2" s="38" t="n"/>
+      <c r="I2" s="38" t="inlineStr">
         <is>
           <t>Last regenerated by tools/update_hotkeys_sheet.py</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="41" t="inlineStr"/>
-      <c r="B3" s="41" t="inlineStr"/>
-      <c r="C3" s="41" t="inlineStr"/>
-      <c r="D3" s="41" t="inlineStr"/>
-      <c r="E3" s="41" t="inlineStr"/>
-      <c r="F3" s="41" t="inlineStr"/>
-      <c r="G3" s="41" t="inlineStr"/>
-      <c r="H3" s="41" t="inlineStr"/>
-      <c r="I3" s="41" t="inlineStr"/>
+      <c r="A3" s="38" t="n"/>
+      <c r="B3" s="38" t="n"/>
+      <c r="C3" s="38" t="n"/>
+      <c r="D3" s="38" t="n"/>
+      <c r="E3" s="38" t="n"/>
+      <c r="F3" s="38" t="n"/>
+      <c r="G3" s="38" t="n"/>
+      <c r="H3" s="38" t="n"/>
+      <c r="I3" s="38" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="42" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>Key / Input</t>
         </is>
       </c>
-      <c r="D4" s="42" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>Modifiers</t>
         </is>
       </c>
-      <c r="E4" s="42" t="inlineStr">
+      <c r="E4" s="39" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="F4" s="42" t="inlineStr">
+      <c r="F4" s="39" t="inlineStr">
         <is>
           <t>Context / Preconditions</t>
         </is>
       </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="G4" s="39" t="inlineStr">
         <is>
           <t>Blocked When</t>
         </is>
       </c>
-      <c r="H4" s="42" t="inlineStr">
+      <c r="H4" s="39" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
       </c>
-      <c r="I4" s="42" t="inlineStr">
+      <c r="I4" s="39" t="inlineStr">
         <is>
           <t>Overlap Notes</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="30" customHeight="1" s="41">
       <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Global</t>
@@ -3179,7 +3329,7 @@
           <t>Space</t>
         </is>
       </c>
-      <c r="D5" s="29" t="inlineStr"/>
+      <c r="D5" s="29" t="n"/>
       <c r="E5" s="29" t="inlineStr">
         <is>
           <t>Toggle simulation pause / resume</t>
@@ -3237,13 +3387,13 @@
           <t>Simulation control active</t>
         </is>
       </c>
-      <c r="G6" s="29" t="inlineStr"/>
+      <c r="G6" s="29" t="n"/>
       <c r="H6" s="29" t="inlineStr">
         <is>
           <t>src/simulation/input.rs</t>
         </is>
       </c>
-      <c r="I6" s="29" t="inlineStr"/>
+      <c r="I6" s="29" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -3261,7 +3411,7 @@
           <t>F12</t>
         </is>
       </c>
-      <c r="D7" s="29" t="inlineStr"/>
+      <c r="D7" s="29" t="n"/>
       <c r="E7" s="29" t="inlineStr">
         <is>
           <t>Toggle Dev Mode on/off</t>
@@ -3272,15 +3422,15 @@
           <t>Always</t>
         </is>
       </c>
-      <c r="G7" s="29" t="inlineStr"/>
+      <c r="G7" s="29" t="n"/>
       <c r="H7" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I7" s="29" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="I7" s="29" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" s="41">
       <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Camera</t>
@@ -3327,7 +3477,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="30" customHeight="1" s="41">
       <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Camera</t>
@@ -3358,7 +3508,7 @@
           <t>While panning</t>
         </is>
       </c>
-      <c r="G9" s="29" t="inlineStr"/>
+      <c r="G9" s="29" t="n"/>
       <c r="H9" s="29" t="inlineStr">
         <is>
           <t>src/camera/control.rs</t>
@@ -3370,7 +3520,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="30" customHeight="1" s="41">
       <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Camera</t>
@@ -3401,13 +3551,13 @@
           <t>Always unless blocked</t>
         </is>
       </c>
-      <c r="G10" s="29" t="inlineStr"/>
+      <c r="G10" s="29" t="n"/>
       <c r="H10" s="29" t="inlineStr">
         <is>
           <t>src/camera/control.rs</t>
         </is>
       </c>
-      <c r="I10" s="29" t="inlineStr"/>
+      <c r="I10" s="29" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -3440,15 +3590,15 @@
           <t>Always unless blocked</t>
         </is>
       </c>
-      <c r="G11" s="29" t="inlineStr"/>
+      <c r="G11" s="29" t="n"/>
       <c r="H11" s="29" t="inlineStr">
         <is>
           <t>src/camera/control.rs</t>
         </is>
       </c>
-      <c r="I11" s="29" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="I11" s="29" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="41">
       <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3489,7 +3639,7 @@
           <t>src/client/pipeline.rs</t>
         </is>
       </c>
-      <c r="I12" s="29" t="inlineStr"/>
+      <c r="I12" s="29" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
@@ -3522,13 +3672,13 @@
           <t>Same as left click path</t>
         </is>
       </c>
-      <c r="G13" s="29" t="inlineStr"/>
+      <c r="G13" s="29" t="n"/>
       <c r="H13" s="29" t="inlineStr">
         <is>
           <t>src/client/pipeline.rs</t>
         </is>
       </c>
-      <c r="I13" s="29" t="inlineStr"/>
+      <c r="I13" s="29" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
@@ -3561,13 +3711,13 @@
           <t>Drag threshold exceeded</t>
         </is>
       </c>
-      <c r="G14" s="29" t="inlineStr"/>
+      <c r="G14" s="29" t="n"/>
       <c r="H14" s="29" t="inlineStr">
         <is>
           <t>src/client/pipeline.rs</t>
         </is>
       </c>
-      <c r="I14" s="29" t="inlineStr"/>
+      <c r="I14" s="29" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
@@ -3600,15 +3750,15 @@
           <t>Box drag</t>
         </is>
       </c>
-      <c r="G15" s="29" t="inlineStr"/>
+      <c r="G15" s="29" t="n"/>
       <c r="H15" s="29" t="inlineStr">
         <is>
           <t>src/client/pipeline.rs</t>
         </is>
       </c>
-      <c r="I15" s="29" t="inlineStr"/>
-    </row>
-    <row r="16">
+      <c r="I15" s="29" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1" s="41">
       <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3639,7 +3789,7 @@
           <t>Unit under cursor</t>
         </is>
       </c>
-      <c r="G16" s="29" t="inlineStr"/>
+      <c r="G16" s="29" t="n"/>
       <c r="H16" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/input.rs</t>
@@ -3651,7 +3801,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="30" customHeight="1" s="41">
       <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3692,9 +3842,9 @@
           <t>src/client/pipeline.rs</t>
         </is>
       </c>
-      <c r="I17" s="29" t="inlineStr"/>
-    </row>
-    <row r="18">
+      <c r="I17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="41">
       <c r="A18" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3710,7 +3860,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D18" s="29" t="inlineStr"/>
+      <c r="D18" s="29" t="n"/>
       <c r="E18" s="29" t="inlineStr">
         <is>
           <t>Enter / exit build mode</t>
@@ -3737,7 +3887,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="30" customHeight="1" s="41">
       <c r="A19" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3753,7 +3903,7 @@
           <t>Esc</t>
         </is>
       </c>
-      <c r="D19" s="29" t="inlineStr"/>
+      <c r="D19" s="29" t="n"/>
       <c r="E19" s="29" t="inlineStr">
         <is>
           <t>Cancel build placement</t>
@@ -3764,7 +3914,7 @@
           <t>Build mode active</t>
         </is>
       </c>
-      <c r="G19" s="29" t="inlineStr"/>
+      <c r="G19" s="29" t="n"/>
       <c r="H19" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/build_mode/input.rs</t>
@@ -3776,7 +3926,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="30" customHeight="1" s="41">
       <c r="A20" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3792,7 +3942,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="D20" s="29" t="inlineStr"/>
+      <c r="D20" s="29" t="n"/>
       <c r="E20" s="29" t="inlineStr">
         <is>
           <t>Rotate build ghost</t>
@@ -3803,7 +3953,7 @@
           <t>Ghost placing</t>
         </is>
       </c>
-      <c r="G20" s="29" t="inlineStr"/>
+      <c r="G20" s="29" t="n"/>
       <c r="H20" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/build_mode/input.rs</t>
@@ -3815,7 +3965,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="30" customHeight="1" s="41">
       <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3846,15 +3996,15 @@
           <t>Build mode active</t>
         </is>
       </c>
-      <c r="G21" s="29" t="inlineStr"/>
+      <c r="G21" s="29" t="n"/>
       <c r="H21" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/build_mode/input.rs</t>
         </is>
       </c>
-      <c r="I21" s="29" t="inlineStr"/>
-    </row>
-    <row r="22">
+      <c r="I21" s="29" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1" s="41">
       <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3885,15 +4035,15 @@
           <t>Ghost placing; valid terrain</t>
         </is>
       </c>
-      <c r="G22" s="29" t="inlineStr"/>
+      <c r="G22" s="29" t="n"/>
       <c r="H22" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/build_mode/input.rs</t>
         </is>
       </c>
-      <c r="I22" s="29" t="inlineStr"/>
-    </row>
-    <row r="23">
+      <c r="I22" s="29" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1" s="41">
       <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3909,7 +4059,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="D23" s="29" t="inlineStr"/>
+      <c r="D23" s="29" t="n"/>
       <c r="E23" s="29" t="inlineStr">
         <is>
           <t>Open primary unit inventory panel</t>
@@ -3920,7 +4070,7 @@
           <t>Primary unit selected</t>
         </is>
       </c>
-      <c r="G23" s="29" t="inlineStr"/>
+      <c r="G23" s="29" t="n"/>
       <c r="H23" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/inventory/input.rs</t>
@@ -3932,7 +4082,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="30" customHeight="1" s="41">
       <c r="A24" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -3948,7 +4098,7 @@
           <t>Esc</t>
         </is>
       </c>
-      <c r="D24" s="29" t="inlineStr"/>
+      <c r="D24" s="29" t="n"/>
       <c r="E24" s="29" t="inlineStr">
         <is>
           <t>Close inventory / cancel drag / cancel split dialog</t>
@@ -3959,13 +4109,13 @@
           <t>Inventory UI open</t>
         </is>
       </c>
-      <c r="G24" s="29" t="inlineStr"/>
+      <c r="G24" s="29" t="n"/>
       <c r="H24" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/inventory/input.rs</t>
         </is>
       </c>
-      <c r="I24" s="29" t="inlineStr"/>
+      <c r="I24" s="29" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
@@ -3998,13 +4148,13 @@
           <t>Inventory open; dual pane</t>
         </is>
       </c>
-      <c r="G25" s="29" t="inlineStr"/>
+      <c r="G25" s="29" t="n"/>
       <c r="H25" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/inventory/panel.rs</t>
         </is>
       </c>
-      <c r="I25" s="29" t="inlineStr"/>
+      <c r="I25" s="29" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
@@ -4037,15 +4187,15 @@
           <t>Inventory open; dual pane</t>
         </is>
       </c>
-      <c r="G26" s="29" t="inlineStr"/>
+      <c r="G26" s="29" t="n"/>
       <c r="H26" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/inventory/panel.rs</t>
         </is>
       </c>
-      <c r="I26" s="29" t="inlineStr"/>
-    </row>
-    <row r="27">
+      <c r="I26" s="29" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1" s="41">
       <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -4061,7 +4211,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D27" s="29" t="inlineStr"/>
+      <c r="D27" s="29" t="n"/>
       <c r="E27" s="29" t="inlineStr">
         <is>
           <t>Toggle Terrain Analysis panel</t>
@@ -4072,7 +4222,7 @@
           <t>Always</t>
         </is>
       </c>
-      <c r="G27" s="29" t="inlineStr"/>
+      <c r="G27" s="29" t="n"/>
       <c r="H27" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/terrain_analysis/mod.rs</t>
@@ -4084,7 +4234,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="30" customHeight="1" s="41">
       <c r="A28" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -4100,7 +4250,7 @@
           <t>[</t>
         </is>
       </c>
-      <c r="D28" s="29" t="inlineStr"/>
+      <c r="D28" s="29" t="n"/>
       <c r="E28" s="29" t="inlineStr">
         <is>
           <t>Decrease overlay opacity</t>
@@ -4111,7 +4261,7 @@
           <t>Terrain Analysis panel open</t>
         </is>
       </c>
-      <c r="G28" s="29" t="inlineStr"/>
+      <c r="G28" s="29" t="n"/>
       <c r="H28" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/terrain_analysis/mod.rs</t>
@@ -4123,7 +4273,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="30" customHeight="1" s="41">
       <c r="A29" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -4139,7 +4289,7 @@
           <t>]</t>
         </is>
       </c>
-      <c r="D29" s="29" t="inlineStr"/>
+      <c r="D29" s="29" t="n"/>
       <c r="E29" s="29" t="inlineStr">
         <is>
           <t>Increase overlay opacity</t>
@@ -4150,7 +4300,7 @@
           <t>Terrain Analysis panel open</t>
         </is>
       </c>
-      <c r="G29" s="29" t="inlineStr"/>
+      <c r="G29" s="29" t="n"/>
       <c r="H29" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/terrain_analysis/mod.rs</t>
@@ -4162,7 +4312,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="30" customHeight="1" s="41">
       <c r="A30" s="29" t="inlineStr">
         <is>
           <t>Gameplay</t>
@@ -4193,7 +4343,7 @@
           <t>Command panel buttons</t>
         </is>
       </c>
-      <c r="G30" s="29" t="inlineStr"/>
+      <c r="G30" s="29" t="n"/>
       <c r="H30" s="29" t="inlineStr">
         <is>
           <t>src/ui/gameplay/command_panel.rs</t>
@@ -4236,13 +4386,13 @@
           <t>Dev mode on</t>
         </is>
       </c>
-      <c r="G31" s="29" t="inlineStr"/>
+      <c r="G31" s="29" t="n"/>
       <c r="H31" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I31" s="29" t="inlineStr"/>
+      <c r="I31" s="29" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
@@ -4260,7 +4410,7 @@
           <t>Tab</t>
         </is>
       </c>
-      <c r="D32" s="29" t="inlineStr"/>
+      <c r="D32" s="29" t="n"/>
       <c r="E32" s="29" t="inlineStr">
         <is>
           <t>Cycle dev panel tabs</t>
@@ -4287,7 +4437,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="30" customHeight="1" s="41">
       <c r="A33" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4303,7 +4453,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="D33" s="29" t="inlineStr"/>
+      <c r="D33" s="29" t="n"/>
       <c r="E33" s="29" t="inlineStr">
         <is>
           <t>Toggle catalog enabled-only filter</t>
@@ -4330,7 +4480,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="30" customHeight="1" s="41">
       <c r="A34" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4346,7 +4496,7 @@
           <t>T</t>
         </is>
       </c>
-      <c r="D34" s="29" t="inlineStr"/>
+      <c r="D34" s="29" t="n"/>
       <c r="E34" s="29" t="inlineStr">
         <is>
           <t>Cycle spawn team (Player ↔ Wilds)</t>
@@ -4373,7 +4523,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="30" customHeight="1" s="41">
       <c r="A35" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4389,7 +4539,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="D35" s="29" t="inlineStr"/>
+      <c r="D35" s="29" t="n"/>
       <c r="E35" s="29" t="inlineStr">
         <is>
           <t>Toggle favorite on selected catalog definition</t>
@@ -4432,7 +4582,7 @@
           <t>1–9</t>
         </is>
       </c>
-      <c r="D36" s="29" t="inlineStr"/>
+      <c r="D36" s="29" t="n"/>
       <c r="E36" s="29" t="inlineStr">
         <is>
           <t>Recall favorite catalog slot</t>
@@ -4500,9 +4650,9 @@
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I37" s="29" t="inlineStr"/>
-    </row>
-    <row r="38">
+      <c r="I37" s="29" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="41">
       <c r="A38" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4518,7 +4668,7 @@
           <t>Esc</t>
         </is>
       </c>
-      <c r="D38" s="29" t="inlineStr"/>
+      <c r="D38" s="29" t="n"/>
       <c r="E38" s="29" t="inlineStr">
         <is>
           <t>Clear text focus; cancel placement tool</t>
@@ -4529,7 +4679,7 @@
           <t>Dev mode on</t>
         </is>
       </c>
-      <c r="G38" s="29" t="inlineStr"/>
+      <c r="G38" s="29" t="n"/>
       <c r="H38" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
@@ -4557,7 +4707,7 @@
           <t>Enter</t>
         </is>
       </c>
-      <c r="D39" s="29" t="inlineStr"/>
+      <c r="D39" s="29" t="n"/>
       <c r="E39" s="29" t="inlineStr">
         <is>
           <t>Exit dev text focus (search, scene name, qty)</t>
@@ -4568,13 +4718,13 @@
           <t>Text field focused</t>
         </is>
       </c>
-      <c r="G39" s="29" t="inlineStr"/>
+      <c r="G39" s="29" t="n"/>
       <c r="H39" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I39" s="29" t="inlineStr"/>
+      <c r="I39" s="29" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="29" t="inlineStr">
@@ -4617,7 +4767,7 @@
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I40" s="29" t="inlineStr"/>
+      <c r="I40" s="29" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
@@ -4650,13 +4800,13 @@
           <t>Placement active</t>
         </is>
       </c>
-      <c r="G41" s="29" t="inlineStr"/>
+      <c r="G41" s="29" t="n"/>
       <c r="H41" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I41" s="29" t="inlineStr"/>
+      <c r="I41" s="29" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="29" t="inlineStr">
@@ -4689,13 +4839,13 @@
           <t>Placement active</t>
         </is>
       </c>
-      <c r="G42" s="29" t="inlineStr"/>
+      <c r="G42" s="29" t="n"/>
       <c r="H42" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I42" s="29" t="inlineStr"/>
+      <c r="I42" s="29" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="29" t="inlineStr">
@@ -4728,15 +4878,15 @@
           <t>Placement armed; not over panel</t>
         </is>
       </c>
-      <c r="G43" s="29" t="inlineStr"/>
+      <c r="G43" s="29" t="n"/>
       <c r="H43" s="29" t="inlineStr">
         <is>
           <t>src/dev/input.rs</t>
         </is>
       </c>
-      <c r="I43" s="29" t="inlineStr"/>
-    </row>
-    <row r="44">
+      <c r="I43" s="29" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1" s="41">
       <c r="A44" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4777,9 +4927,9 @@
           <t>src/dev/inspector/input.rs</t>
         </is>
       </c>
-      <c r="I44" s="29" t="inlineStr"/>
-    </row>
-    <row r="45">
+      <c r="I44" s="29" t="n"/>
+    </row>
+    <row r="45" ht="30" customHeight="1" s="41">
       <c r="A45" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4795,7 +4945,7 @@
           <t>,</t>
         </is>
       </c>
-      <c r="D45" s="29" t="inlineStr"/>
+      <c r="D45" s="29" t="n"/>
       <c r="E45" s="29" t="inlineStr">
         <is>
           <t>Translate gizmo mode</t>
@@ -4822,7 +4972,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="30" customHeight="1" s="41">
       <c r="A46" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4838,7 +4988,7 @@
           <t>.</t>
         </is>
       </c>
-      <c r="D46" s="29" t="inlineStr"/>
+      <c r="D46" s="29" t="n"/>
       <c r="E46" s="29" t="inlineStr">
         <is>
           <t>Rotate gizmo mode</t>
@@ -4865,7 +5015,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="30" customHeight="1" s="41">
       <c r="A47" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -4881,7 +5031,7 @@
           <t>/</t>
         </is>
       </c>
-      <c r="D47" s="29" t="inlineStr"/>
+      <c r="D47" s="29" t="n"/>
       <c r="E47" s="29" t="inlineStr">
         <is>
           <t>Scale gizmo mode</t>
@@ -4924,7 +5074,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D48" s="29" t="inlineStr"/>
+      <c r="D48" s="29" t="n"/>
       <c r="E48" s="29" t="inlineStr">
         <is>
           <t>Toggle world/local coordinate space</t>
@@ -4935,7 +5085,7 @@
           <t>Gizmo dragging</t>
         </is>
       </c>
-      <c r="G48" s="29" t="inlineStr"/>
+      <c r="G48" s="29" t="n"/>
       <c r="H48" s="29" t="inlineStr">
         <is>
           <t>src/dev/gizmo/input.rs</t>
@@ -4963,7 +5113,7 @@
           <t>X / Y / Z</t>
         </is>
       </c>
-      <c r="D49" s="29" t="inlineStr"/>
+      <c r="D49" s="29" t="n"/>
       <c r="E49" s="29" t="inlineStr">
         <is>
           <t>Axis constraint while dragging</t>
@@ -4974,7 +5124,7 @@
           <t>Gizmo drag active</t>
         </is>
       </c>
-      <c r="G49" s="29" t="inlineStr"/>
+      <c r="G49" s="29" t="n"/>
       <c r="H49" s="29" t="inlineStr">
         <is>
           <t>src/dev/gizmo/input.rs</t>
@@ -5002,7 +5152,7 @@
           <t>Esc</t>
         </is>
       </c>
-      <c r="D50" s="29" t="inlineStr"/>
+      <c r="D50" s="29" t="n"/>
       <c r="E50" s="29" t="inlineStr">
         <is>
           <t>Cancel gizmo drag or exit transform mode</t>
@@ -5013,13 +5163,13 @@
           <t>Gizmo active</t>
         </is>
       </c>
-      <c r="G50" s="29" t="inlineStr"/>
+      <c r="G50" s="29" t="n"/>
       <c r="H50" s="29" t="inlineStr">
         <is>
           <t>src/dev/gizmo/input.rs</t>
         </is>
       </c>
-      <c r="I50" s="29" t="inlineStr"/>
+      <c r="I50" s="29" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="29" t="inlineStr">
@@ -5052,7 +5202,7 @@
           <t>Committing transform</t>
         </is>
       </c>
-      <c r="G51" s="29" t="inlineStr"/>
+      <c r="G51" s="29" t="n"/>
       <c r="H51" s="29" t="inlineStr">
         <is>
           <t>src/dev/gizmo/commit.rs</t>
@@ -5064,7 +5214,7 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="30" customHeight="1" s="41">
       <c r="A52" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5095,15 +5245,15 @@
           <t>Committing doodad/building transform</t>
         </is>
       </c>
-      <c r="G52" s="29" t="inlineStr"/>
+      <c r="G52" s="29" t="n"/>
       <c r="H52" s="29" t="inlineStr">
         <is>
           <t>src/dev/gizmo/commit.rs</t>
         </is>
       </c>
-      <c r="I52" s="29" t="inlineStr"/>
-    </row>
-    <row r="53">
+      <c r="I52" s="29" t="n"/>
+    </row>
+    <row r="53" ht="30" customHeight="1" s="41">
       <c r="A53" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5134,15 +5284,15 @@
           <t>Building gizmo commit</t>
         </is>
       </c>
-      <c r="G53" s="29" t="inlineStr"/>
+      <c r="G53" s="29" t="n"/>
       <c r="H53" s="29" t="inlineStr">
         <is>
           <t>src/dev/gizmo/commit.rs</t>
         </is>
       </c>
-      <c r="I53" s="29" t="inlineStr"/>
-    </row>
-    <row r="54">
+      <c r="I53" s="29" t="n"/>
+    </row>
+    <row r="54" ht="30" customHeight="1" s="41">
       <c r="A54" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5158,7 +5308,7 @@
           <t>Arrow keys</t>
         </is>
       </c>
-      <c r="D54" s="29" t="inlineStr"/>
+      <c r="D54" s="29" t="n"/>
       <c r="E54" s="29" t="inlineStr">
         <is>
           <t>Move doodad X/Z</t>
@@ -5179,9 +5329,9 @@
           <t>src/dev/inspector/doodad_actions.rs</t>
         </is>
       </c>
-      <c r="I54" s="29" t="inlineStr"/>
-    </row>
-    <row r="55">
+      <c r="I54" s="29" t="n"/>
+    </row>
+    <row r="55" ht="30" customHeight="1" s="41">
       <c r="A55" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5197,7 +5347,7 @@
           <t>Page Up / Down</t>
         </is>
       </c>
-      <c r="D55" s="29" t="inlineStr"/>
+      <c r="D55" s="29" t="n"/>
       <c r="E55" s="29" t="inlineStr">
         <is>
           <t>Move doodad Y</t>
@@ -5208,15 +5358,15 @@
           <t>Doodad selected</t>
         </is>
       </c>
-      <c r="G55" s="29" t="inlineStr"/>
+      <c r="G55" s="29" t="n"/>
       <c r="H55" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/doodad_actions.rs</t>
         </is>
       </c>
-      <c r="I55" s="29" t="inlineStr"/>
-    </row>
-    <row r="56">
+      <c r="I55" s="29" t="n"/>
+    </row>
+    <row r="56" ht="30" customHeight="1" s="41">
       <c r="A56" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5232,7 +5382,7 @@
           <t>[ / ]</t>
         </is>
       </c>
-      <c r="D56" s="29" t="inlineStr"/>
+      <c r="D56" s="29" t="n"/>
       <c r="E56" s="29" t="inlineStr">
         <is>
           <t>Adjust doodad yaw ±5°</t>
@@ -5243,7 +5393,7 @@
           <t>Doodad selected</t>
         </is>
       </c>
-      <c r="G56" s="29" t="inlineStr"/>
+      <c r="G56" s="29" t="n"/>
       <c r="H56" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/doodad_actions.rs</t>
@@ -5255,7 +5405,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="30" customHeight="1" s="41">
       <c r="A57" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5286,15 +5436,15 @@
           <t>While applying doodad edit</t>
         </is>
       </c>
-      <c r="G57" s="29" t="inlineStr"/>
+      <c r="G57" s="29" t="n"/>
       <c r="H57" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/doodad_actions.rs</t>
         </is>
       </c>
-      <c r="I57" s="29" t="inlineStr"/>
-    </row>
-    <row r="58">
+      <c r="I57" s="29" t="n"/>
+    </row>
+    <row r="58" ht="30" customHeight="1" s="41">
       <c r="A58" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5325,15 +5475,15 @@
           <t>While applying doodad edit</t>
         </is>
       </c>
-      <c r="G58" s="29" t="inlineStr"/>
+      <c r="G58" s="29" t="n"/>
       <c r="H58" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/doodad_actions.rs</t>
         </is>
       </c>
-      <c r="I58" s="29" t="inlineStr"/>
-    </row>
-    <row r="59">
+      <c r="I58" s="29" t="n"/>
+    </row>
+    <row r="59" ht="30" customHeight="1" s="41">
       <c r="A59" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5349,7 +5499,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="D59" s="29" t="inlineStr"/>
+      <c r="D59" s="29" t="n"/>
       <c r="E59" s="29" t="inlineStr">
         <is>
           <t>Damage building (−50)</t>
@@ -5370,9 +5520,9 @@
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I59" s="29" t="inlineStr"/>
-    </row>
-    <row r="60">
+      <c r="I59" s="29" t="n"/>
+    </row>
+    <row r="60" ht="30" customHeight="1" s="41">
       <c r="A60" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5388,7 +5538,7 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D60" s="29" t="inlineStr"/>
+      <c r="D60" s="29" t="n"/>
       <c r="E60" s="29" t="inlineStr">
         <is>
           <t>Heal building (+50)</t>
@@ -5399,7 +5549,7 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G60" s="29" t="inlineStr"/>
+      <c r="G60" s="29" t="n"/>
       <c r="H60" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -5411,7 +5561,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="30" customHeight="1" s="41">
       <c r="A61" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5427,7 +5577,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="D61" s="29" t="inlineStr"/>
+      <c r="D61" s="29" t="n"/>
       <c r="E61" s="29" t="inlineStr">
         <is>
           <t>Destroy building</t>
@@ -5438,15 +5588,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G61" s="29" t="inlineStr"/>
+      <c r="G61" s="29" t="n"/>
       <c r="H61" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I61" s="29" t="inlineStr"/>
-    </row>
-    <row r="62">
+      <c r="I61" s="29" t="n"/>
+    </row>
+    <row r="62" ht="30" customHeight="1" s="41">
       <c r="A62" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5462,7 +5612,7 @@
           <t>R</t>
         </is>
       </c>
-      <c r="D62" s="29" t="inlineStr"/>
+      <c r="D62" s="29" t="n"/>
       <c r="E62" s="29" t="inlineStr">
         <is>
           <t>Set building to ruins</t>
@@ -5473,7 +5623,7 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G62" s="29" t="inlineStr"/>
+      <c r="G62" s="29" t="n"/>
       <c r="H62" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -5485,7 +5635,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="30" customHeight="1" s="41">
       <c r="A63" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5501,7 +5651,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D63" s="29" t="inlineStr"/>
+      <c r="D63" s="29" t="n"/>
       <c r="E63" s="29" t="inlineStr">
         <is>
           <t>Complete building (lifecycle)</t>
@@ -5512,15 +5662,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G63" s="29" t="inlineStr"/>
+      <c r="G63" s="29" t="n"/>
       <c r="H63" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I63" s="29" t="inlineStr"/>
-    </row>
-    <row r="64">
+      <c r="I63" s="29" t="n"/>
+    </row>
+    <row r="64" ht="30" customHeight="1" s="41">
       <c r="A64" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5536,7 +5686,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D64" s="29" t="inlineStr"/>
+      <c r="D64" s="29" t="n"/>
       <c r="E64" s="29" t="inlineStr">
         <is>
           <t>Add 10% construction progress</t>
@@ -5547,7 +5697,7 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G64" s="29" t="inlineStr"/>
+      <c r="G64" s="29" t="n"/>
       <c r="H64" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -5559,7 +5709,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="30" customHeight="1" s="41">
       <c r="A65" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5590,15 +5740,15 @@
           <t>Building linked to settlement</t>
         </is>
       </c>
-      <c r="G65" s="29" t="inlineStr"/>
+      <c r="G65" s="29" t="n"/>
       <c r="H65" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I65" s="29" t="inlineStr"/>
-    </row>
-    <row r="66">
+      <c r="I65" s="29" t="n"/>
+    </row>
+    <row r="66" ht="30" customHeight="1" s="41">
       <c r="A66" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5614,7 +5764,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="D66" s="29" t="inlineStr"/>
+      <c r="D66" s="29" t="n"/>
       <c r="E66" s="29" t="inlineStr">
         <is>
           <t>Open first building door</t>
@@ -5625,15 +5775,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G66" s="29" t="inlineStr"/>
+      <c r="G66" s="29" t="n"/>
       <c r="H66" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I66" s="29" t="inlineStr"/>
-    </row>
-    <row r="67">
+      <c r="I66" s="29" t="n"/>
+    </row>
+    <row r="67" ht="30" customHeight="1" s="41">
       <c r="A67" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5649,7 +5799,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="D67" s="29" t="inlineStr"/>
+      <c r="D67" s="29" t="n"/>
       <c r="E67" s="29" t="inlineStr">
         <is>
           <t>Lock first building door</t>
@@ -5660,15 +5810,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G67" s="29" t="inlineStr"/>
+      <c r="G67" s="29" t="n"/>
       <c r="H67" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I67" s="29" t="inlineStr"/>
-    </row>
-    <row r="68">
+      <c r="I67" s="29" t="n"/>
+    </row>
+    <row r="68" ht="30" customHeight="1" s="41">
       <c r="A68" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5684,7 +5834,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="D68" s="29" t="inlineStr"/>
+      <c r="D68" s="29" t="n"/>
       <c r="E68" s="29" t="inlineStr">
         <is>
           <t>Log building inventory summary</t>
@@ -5695,7 +5845,7 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G68" s="29" t="inlineStr"/>
+      <c r="G68" s="29" t="n"/>
       <c r="H68" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -5707,7 +5857,7 @@
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="30" customHeight="1" s="41">
       <c r="A69" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5723,7 +5873,7 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D69" s="29" t="inlineStr"/>
+      <c r="D69" s="29" t="n"/>
       <c r="E69" s="29" t="inlineStr">
         <is>
           <t>Add 5 gold to building inventory</t>
@@ -5734,15 +5884,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G69" s="29" t="inlineStr"/>
+      <c r="G69" s="29" t="n"/>
       <c r="H69" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I69" s="29" t="inlineStr"/>
-    </row>
-    <row r="70">
+      <c r="I69" s="29" t="n"/>
+    </row>
+    <row r="70" ht="30" customHeight="1" s="41">
       <c r="A70" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5758,7 +5908,7 @@
           <t>T</t>
         </is>
       </c>
-      <c r="D70" s="29" t="inlineStr"/>
+      <c r="D70" s="29" t="n"/>
       <c r="E70" s="29" t="inlineStr">
         <is>
           <t>Transfer item between selected unit and building</t>
@@ -5769,15 +5919,15 @@
           <t>Unit + building with inventories</t>
         </is>
       </c>
-      <c r="G70" s="29" t="inlineStr"/>
+      <c r="G70" s="29" t="n"/>
       <c r="H70" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I70" s="29" t="inlineStr"/>
-    </row>
-    <row r="71">
+      <c r="I70" s="29" t="n"/>
+    </row>
+    <row r="71" ht="30" customHeight="1" s="41">
       <c r="A71" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5793,7 +5943,7 @@
           <t>U</t>
         </is>
       </c>
-      <c r="D71" s="29" t="inlineStr"/>
+      <c r="D71" s="29" t="n"/>
       <c r="E71" s="29" t="inlineStr">
         <is>
           <t>Toggle building container locked</t>
@@ -5804,15 +5954,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G71" s="29" t="inlineStr"/>
+      <c r="G71" s="29" t="n"/>
       <c r="H71" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I71" s="29" t="inlineStr"/>
-    </row>
-    <row r="72">
+      <c r="I71" s="29" t="n"/>
+    </row>
+    <row r="72" ht="30" customHeight="1" s="41">
       <c r="A72" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5828,7 +5978,7 @@
           <t>V</t>
         </is>
       </c>
-      <c r="D72" s="29" t="inlineStr"/>
+      <c r="D72" s="29" t="n"/>
       <c r="E72" s="29" t="inlineStr">
         <is>
           <t>Validate building inventory links</t>
@@ -5839,15 +5989,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G72" s="29" t="inlineStr"/>
+      <c r="G72" s="29" t="n"/>
       <c r="H72" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I72" s="29" t="inlineStr"/>
-    </row>
-    <row r="73">
+      <c r="I72" s="29" t="n"/>
+    </row>
+    <row r="73" ht="30" customHeight="1" s="41">
       <c r="A73" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5863,7 +6013,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="D73" s="29" t="inlineStr"/>
+      <c r="D73" s="29" t="n"/>
       <c r="E73" s="29" t="inlineStr">
         <is>
           <t>Refresh building terrain assessment</t>
@@ -5874,15 +6024,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G73" s="29" t="inlineStr"/>
+      <c r="G73" s="29" t="n"/>
       <c r="H73" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I73" s="29" t="inlineStr"/>
-    </row>
-    <row r="74">
+      <c r="I73" s="29" t="n"/>
+    </row>
+    <row r="74" ht="30" customHeight="1" s="41">
       <c r="A74" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5898,7 +6048,7 @@
           <t>,</t>
         </is>
       </c>
-      <c r="D74" s="29" t="inlineStr"/>
+      <c r="D74" s="29" t="n"/>
       <c r="E74" s="29" t="inlineStr">
         <is>
           <t>Toggle production enabled</t>
@@ -5909,7 +6059,7 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G74" s="29" t="inlineStr"/>
+      <c r="G74" s="29" t="n"/>
       <c r="H74" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -5921,7 +6071,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="30" customHeight="1" s="41">
       <c r="A75" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5937,7 +6087,7 @@
           <t>.</t>
         </is>
       </c>
-      <c r="D75" s="29" t="inlineStr"/>
+      <c r="D75" s="29" t="n"/>
       <c r="E75" s="29" t="inlineStr">
         <is>
           <t>Toggle production paused</t>
@@ -5948,7 +6098,7 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G75" s="29" t="inlineStr"/>
+      <c r="G75" s="29" t="n"/>
       <c r="H75" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -5960,7 +6110,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="30" customHeight="1" s="41">
       <c r="A76" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -5976,7 +6126,7 @@
           <t>]</t>
         </is>
       </c>
-      <c r="D76" s="29" t="inlineStr"/>
+      <c r="D76" s="29" t="n"/>
       <c r="E76" s="29" t="inlineStr">
         <is>
           <t>Reset production progress</t>
@@ -5987,15 +6137,15 @@
           <t>Building selected; blueprint inspection inactive</t>
         </is>
       </c>
-      <c r="G76" s="29" t="inlineStr"/>
+      <c r="G76" s="29" t="n"/>
       <c r="H76" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I76" s="29" t="inlineStr"/>
-    </row>
-    <row r="77">
+      <c r="I76" s="29" t="n"/>
+    </row>
+    <row r="77" ht="30" customHeight="1" s="41">
       <c r="A77" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6011,7 +6161,7 @@
           <t>`</t>
         </is>
       </c>
-      <c r="D77" s="29" t="inlineStr"/>
+      <c r="D77" s="29" t="n"/>
       <c r="E77" s="29" t="inlineStr">
         <is>
           <t>Toggle production advanced panel</t>
@@ -6022,15 +6172,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G77" s="29" t="inlineStr"/>
+      <c r="G77" s="29" t="n"/>
       <c r="H77" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I77" s="29" t="inlineStr"/>
-    </row>
-    <row r="78">
+      <c r="I77" s="29" t="n"/>
+    </row>
+    <row r="78" ht="30" customHeight="1" s="41">
       <c r="A78" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6046,7 +6196,7 @@
           <t>\</t>
         </is>
       </c>
-      <c r="D78" s="29" t="inlineStr"/>
+      <c r="D78" s="29" t="n"/>
       <c r="E78" s="29" t="inlineStr">
         <is>
           <t>Validate production runtime</t>
@@ -6057,15 +6207,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G78" s="29" t="inlineStr"/>
+      <c r="G78" s="29" t="n"/>
       <c r="H78" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I78" s="29" t="inlineStr"/>
-    </row>
-    <row r="79">
+      <c r="I78" s="29" t="n"/>
+    </row>
+    <row r="79" ht="30" customHeight="1" s="41">
       <c r="A79" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6081,7 +6231,7 @@
           <t>'</t>
         </is>
       </c>
-      <c r="D79" s="29" t="inlineStr"/>
+      <c r="D79" s="29" t="n"/>
       <c r="E79" s="29" t="inlineStr">
         <is>
           <t>Cycle production operation (forward)</t>
@@ -6092,15 +6242,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G79" s="29" t="inlineStr"/>
+      <c r="G79" s="29" t="n"/>
       <c r="H79" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I79" s="29" t="inlineStr"/>
-    </row>
-    <row r="80">
+      <c r="I79" s="29" t="n"/>
+    </row>
+    <row r="80" ht="30" customHeight="1" s="41">
       <c r="A80" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6116,7 +6266,7 @@
           <t>;</t>
         </is>
       </c>
-      <c r="D80" s="29" t="inlineStr"/>
+      <c r="D80" s="29" t="n"/>
       <c r="E80" s="29" t="inlineStr">
         <is>
           <t>Cycle production operation (backward)</t>
@@ -6127,15 +6277,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G80" s="29" t="inlineStr"/>
+      <c r="G80" s="29" t="n"/>
       <c r="H80" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I80" s="29" t="inlineStr"/>
-    </row>
-    <row r="81">
+      <c r="I80" s="29" t="n"/>
+    </row>
+    <row r="81" ht="30" customHeight="1" s="41">
       <c r="A81" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6151,7 +6301,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D81" s="29" t="inlineStr"/>
+      <c r="D81" s="29" t="n"/>
       <c r="E81" s="29" t="inlineStr">
         <is>
           <t>Force-execute one production cycle</t>
@@ -6162,15 +6312,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G81" s="29" t="inlineStr"/>
+      <c r="G81" s="29" t="n"/>
       <c r="H81" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I81" s="29" t="inlineStr"/>
-    </row>
-    <row r="82">
+      <c r="I81" s="29" t="n"/>
+    </row>
+    <row r="82" ht="30" customHeight="1" s="41">
       <c r="A82" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6186,7 +6336,7 @@
           <t>K</t>
         </is>
       </c>
-      <c r="D82" s="29" t="inlineStr"/>
+      <c r="D82" s="29" t="n"/>
       <c r="E82" s="29" t="inlineStr">
         <is>
           <t>Clear binding inventories</t>
@@ -6197,15 +6347,15 @@
           <t>Building selected</t>
         </is>
       </c>
-      <c r="G82" s="29" t="inlineStr"/>
+      <c r="G82" s="29" t="n"/>
       <c r="H82" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I82" s="29" t="inlineStr"/>
-    </row>
-    <row r="83">
+      <c r="I82" s="29" t="n"/>
+    </row>
+    <row r="83" ht="30" customHeight="1" s="41">
       <c r="A83" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6221,7 +6371,7 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="D83" s="29" t="inlineStr"/>
+      <c r="D83" s="29" t="n"/>
       <c r="E83" s="29" t="inlineStr">
         <is>
           <t>Spawn manual haul / cancel hauls / force-complete (modifiers)</t>
@@ -6232,15 +6382,15 @@
           <t>Building selected; Shift=cancel open; Ctrl=force complete</t>
         </is>
       </c>
-      <c r="G83" s="29" t="inlineStr"/>
+      <c r="G83" s="29" t="n"/>
       <c r="H83" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
         </is>
       </c>
-      <c r="I83" s="29" t="inlineStr"/>
-    </row>
-    <row r="84">
+      <c r="I83" s="29" t="n"/>
+    </row>
+    <row r="84" ht="30" customHeight="1" s="41">
       <c r="A84" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6271,7 +6421,7 @@
           <t>Building selected; Inspector tab</t>
         </is>
       </c>
-      <c r="G84" s="29" t="inlineStr"/>
+      <c r="G84" s="29" t="n"/>
       <c r="H84" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/building_actions.rs</t>
@@ -6283,7 +6433,7 @@
         </is>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="30" customHeight="1" s="41">
       <c r="A85" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6299,7 +6449,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="D85" s="29" t="inlineStr"/>
+      <c r="D85" s="29" t="n"/>
       <c r="E85" s="29" t="inlineStr">
         <is>
           <t>Enter blueprint inspection mode</t>
@@ -6310,15 +6460,15 @@
           <t>Building selected; not already inspecting</t>
         </is>
       </c>
-      <c r="G85" s="29" t="inlineStr"/>
+      <c r="G85" s="29" t="n"/>
       <c r="H85" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_inspection.rs</t>
         </is>
       </c>
-      <c r="I85" s="29" t="inlineStr"/>
-    </row>
-    <row r="86">
+      <c r="I85" s="29" t="n"/>
+    </row>
+    <row r="86" ht="30" customHeight="1" s="41">
       <c r="A86" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6334,7 +6484,7 @@
           <t>Esc</t>
         </is>
       </c>
-      <c r="D86" s="29" t="inlineStr"/>
+      <c r="D86" s="29" t="n"/>
       <c r="E86" s="29" t="inlineStr">
         <is>
           <t>Exit blueprint inspection</t>
@@ -6345,15 +6495,15 @@
           <t>Inspection active; not editing</t>
         </is>
       </c>
-      <c r="G86" s="29" t="inlineStr"/>
+      <c r="G86" s="29" t="n"/>
       <c r="H86" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_inspection.rs</t>
         </is>
       </c>
-      <c r="I86" s="29" t="inlineStr"/>
-    </row>
-    <row r="87">
+      <c r="I86" s="29" t="n"/>
+    </row>
+    <row r="87" ht="30" customHeight="1" s="41">
       <c r="A87" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6369,7 +6519,7 @@
           <t>[ / ]</t>
         </is>
       </c>
-      <c r="D87" s="29" t="inlineStr"/>
+      <c r="D87" s="29" t="n"/>
       <c r="E87" s="29" t="inlineStr">
         <is>
           <t>Previous / next floor</t>
@@ -6380,15 +6530,15 @@
           <t>Inspection active</t>
         </is>
       </c>
-      <c r="G87" s="29" t="inlineStr"/>
+      <c r="G87" s="29" t="n"/>
       <c r="H87" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_inspection.rs</t>
         </is>
       </c>
-      <c r="I87" s="29" t="inlineStr"/>
-    </row>
-    <row r="88">
+      <c r="I87" s="29" t="n"/>
+    </row>
+    <row r="88" ht="30" customHeight="1" s="41">
       <c r="A88" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6419,15 +6569,15 @@
           <t>Inspection active</t>
         </is>
       </c>
-      <c r="G88" s="29" t="inlineStr"/>
+      <c r="G88" s="29" t="n"/>
       <c r="H88" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_inspection.rs</t>
         </is>
       </c>
-      <c r="I88" s="29" t="inlineStr"/>
-    </row>
-    <row r="89">
+      <c r="I88" s="29" t="n"/>
+    </row>
+    <row r="89" ht="30" customHeight="1" s="41">
       <c r="A89" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6443,7 +6593,7 @@
           <t>1–9</t>
         </is>
       </c>
-      <c r="D89" s="29" t="inlineStr"/>
+      <c r="D89" s="29" t="n"/>
       <c r="E89" s="29" t="inlineStr">
         <is>
           <t>Focus validation diagnostic N</t>
@@ -6454,7 +6604,7 @@
           <t>Inspection active</t>
         </is>
       </c>
-      <c r="G89" s="29" t="inlineStr"/>
+      <c r="G89" s="29" t="n"/>
       <c r="H89" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_inspection.rs</t>
@@ -6466,7 +6616,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="30" customHeight="1" s="41">
       <c r="A90" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -6482,7 +6632,7 @@
           <t>Enter / Esc</t>
         </is>
       </c>
-      <c r="D90" s="29" t="inlineStr"/>
+      <c r="D90" s="29" t="n"/>
       <c r="E90" s="29" t="inlineStr">
         <is>
           <t>Confirm / cancel pending blueprint action</t>
@@ -6493,13 +6643,13 @@
           <t>Pending confirmation dialog</t>
         </is>
       </c>
-      <c r="G90" s="29" t="inlineStr"/>
+      <c r="G90" s="29" t="n"/>
       <c r="H90" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_inspection.rs</t>
         </is>
       </c>
-      <c r="I90" s="29" t="inlineStr"/>
+      <c r="I90" s="29" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="29" t="inlineStr">
@@ -6517,7 +6667,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="D91" s="29" t="inlineStr"/>
+      <c r="D91" s="29" t="n"/>
       <c r="E91" s="29" t="inlineStr">
         <is>
           <t>Enter blueprint edit mode</t>
@@ -6528,7 +6678,7 @@
           <t>Building selected; not editing</t>
         </is>
       </c>
-      <c r="G91" s="29" t="inlineStr"/>
+      <c r="G91" s="29" t="n"/>
       <c r="H91" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
@@ -6571,13 +6721,13 @@
           <t>Edit mode</t>
         </is>
       </c>
-      <c r="G92" s="29" t="inlineStr"/>
+      <c r="G92" s="29" t="n"/>
       <c r="H92" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I92" s="29" t="inlineStr"/>
+      <c r="I92" s="29" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="29" t="inlineStr">
@@ -6610,13 +6760,13 @@
           <t>Edit mode</t>
         </is>
       </c>
-      <c r="G93" s="29" t="inlineStr"/>
+      <c r="G93" s="29" t="n"/>
       <c r="H93" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I93" s="29" t="inlineStr"/>
+      <c r="I93" s="29" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="29" t="inlineStr">
@@ -6649,13 +6799,13 @@
           <t>Edit mode</t>
         </is>
       </c>
-      <c r="G94" s="29" t="inlineStr"/>
+      <c r="G94" s="29" t="n"/>
       <c r="H94" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I94" s="29" t="inlineStr"/>
+      <c r="I94" s="29" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="29" t="inlineStr">
@@ -6688,13 +6838,13 @@
           <t>Edit mode</t>
         </is>
       </c>
-      <c r="G95" s="29" t="inlineStr"/>
+      <c r="G95" s="29" t="n"/>
       <c r="H95" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I95" s="29" t="inlineStr"/>
+      <c r="I95" s="29" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="29" t="inlineStr">
@@ -6712,7 +6862,7 @@
           <t>1 / 2 / 3</t>
         </is>
       </c>
-      <c r="D96" s="29" t="inlineStr"/>
+      <c r="D96" s="29" t="n"/>
       <c r="E96" s="29" t="inlineStr">
         <is>
           <t>Edit tool: select / add vertex / add entrance</t>
@@ -6723,13 +6873,13 @@
           <t>Edit mode</t>
         </is>
       </c>
-      <c r="G96" s="29" t="inlineStr"/>
+      <c r="G96" s="29" t="n"/>
       <c r="H96" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I96" s="29" t="inlineStr"/>
+      <c r="I96" s="29" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="29" t="inlineStr">
@@ -6747,7 +6897,7 @@
           <t>Del / Backspace</t>
         </is>
       </c>
-      <c r="D97" s="29" t="inlineStr"/>
+      <c r="D97" s="29" t="n"/>
       <c r="E97" s="29" t="inlineStr">
         <is>
           <t>Delete selected blueprint element</t>
@@ -6758,13 +6908,13 @@
           <t>Edit mode</t>
         </is>
       </c>
-      <c r="G97" s="29" t="inlineStr"/>
+      <c r="G97" s="29" t="n"/>
       <c r="H97" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I97" s="29" t="inlineStr"/>
+      <c r="I97" s="29" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="29" t="inlineStr">
@@ -6782,7 +6932,7 @@
           <t>+ / -</t>
         </is>
       </c>
-      <c r="D98" s="29" t="inlineStr"/>
+      <c r="D98" s="29" t="n"/>
       <c r="E98" s="29" t="inlineStr">
         <is>
           <t>Adjust entrance/transition radius</t>
@@ -6793,13 +6943,13 @@
           <t>Edit mode; element selected</t>
         </is>
       </c>
-      <c r="G98" s="29" t="inlineStr"/>
+      <c r="G98" s="29" t="n"/>
       <c r="H98" s="29" t="inlineStr">
         <is>
           <t>src/dev/inspector/blueprint_edit.rs</t>
         </is>
       </c>
-      <c r="I98" s="29" t="inlineStr"/>
+      <c r="I98" s="29" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="29" t="inlineStr">
@@ -6817,7 +6967,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="D99" s="29" t="inlineStr"/>
+      <c r="D99" s="29" t="n"/>
       <c r="E99" s="29" t="inlineStr">
         <is>
           <t>Switch to Items subtab</t>
@@ -6838,7 +6988,7 @@
           <t>src/dev/inventory_tools/input.rs</t>
         </is>
       </c>
-      <c r="I99" s="29" t="inlineStr"/>
+      <c r="I99" s="29" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="29" t="inlineStr">
@@ -6856,7 +7006,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D100" s="29" t="inlineStr"/>
+      <c r="D100" s="29" t="n"/>
       <c r="E100" s="29" t="inlineStr">
         <is>
           <t>Switch to Inventory Profiles subtab</t>
@@ -6867,13 +7017,13 @@
           <t>Items tab</t>
         </is>
       </c>
-      <c r="G100" s="29" t="inlineStr"/>
+      <c r="G100" s="29" t="n"/>
       <c r="H100" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
         </is>
       </c>
-      <c r="I100" s="29" t="inlineStr"/>
+      <c r="I100" s="29" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="29" t="inlineStr">
@@ -6891,7 +7041,7 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D101" s="29" t="inlineStr"/>
+      <c r="D101" s="29" t="n"/>
       <c r="E101" s="29" t="inlineStr">
         <is>
           <t>Switch to Inventory Manage subtab</t>
@@ -6902,13 +7052,13 @@
           <t>Items tab</t>
         </is>
       </c>
-      <c r="G101" s="29" t="inlineStr"/>
+      <c r="G101" s="29" t="n"/>
       <c r="H101" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
         </is>
       </c>
-      <c r="I101" s="29" t="inlineStr"/>
+      <c r="I101" s="29" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="29" t="inlineStr">
@@ -6926,7 +7076,7 @@
           <t>[ / ]</t>
         </is>
       </c>
-      <c r="D102" s="29" t="inlineStr"/>
+      <c r="D102" s="29" t="n"/>
       <c r="E102" s="29" t="inlineStr">
         <is>
           <t>Divide / multiply quantity by 10</t>
@@ -6937,13 +7087,13 @@
           <t>Manage subtab</t>
         </is>
       </c>
-      <c r="G102" s="29" t="inlineStr"/>
+      <c r="G102" s="29" t="n"/>
       <c r="H102" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
         </is>
       </c>
-      <c r="I102" s="29" t="inlineStr"/>
+      <c r="I102" s="29" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="29" t="inlineStr">
@@ -6961,7 +7111,7 @@
           <t>+ / -</t>
         </is>
       </c>
-      <c r="D103" s="29" t="inlineStr"/>
+      <c r="D103" s="29" t="n"/>
       <c r="E103" s="29" t="inlineStr">
         <is>
           <t>Increment / decrement quantity</t>
@@ -6972,13 +7122,13 @@
           <t>Manage subtab</t>
         </is>
       </c>
-      <c r="G103" s="29" t="inlineStr"/>
+      <c r="G103" s="29" t="n"/>
       <c r="H103" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
         </is>
       </c>
-      <c r="I103" s="29" t="inlineStr"/>
+      <c r="I103" s="29" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="29" t="inlineStr">
@@ -6996,7 +7146,7 @@
           <t>T</t>
         </is>
       </c>
-      <c r="D104" s="29" t="inlineStr"/>
+      <c r="D104" s="29" t="n"/>
       <c r="E104" s="29" t="inlineStr">
         <is>
           <t>Cycle inventory endpoint</t>
@@ -7007,7 +7157,7 @@
           <t>Manage subtab</t>
         </is>
       </c>
-      <c r="G104" s="29" t="inlineStr"/>
+      <c r="G104" s="29" t="n"/>
       <c r="H104" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
@@ -7035,7 +7185,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D105" s="29" t="inlineStr"/>
+      <c r="D105" s="29" t="n"/>
       <c r="E105" s="29" t="inlineStr">
         <is>
           <t>Cycle entry within endpoint</t>
@@ -7046,15 +7196,15 @@
           <t>Manage subtab</t>
         </is>
       </c>
-      <c r="G105" s="29" t="inlineStr"/>
+      <c r="G105" s="29" t="n"/>
       <c r="H105" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
         </is>
       </c>
-      <c r="I105" s="29" t="inlineStr"/>
-    </row>
-    <row r="106">
+      <c r="I105" s="29" t="n"/>
+    </row>
+    <row r="106" ht="30" customHeight="1" s="41">
       <c r="A106" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -7070,7 +7220,7 @@
           <t>A / R / S / C / F / G / V</t>
         </is>
       </c>
-      <c r="D106" s="29" t="inlineStr"/>
+      <c r="D106" s="29" t="n"/>
       <c r="E106" s="29" t="inlineStr">
         <is>
           <t>Add / remove / set qty / clear / fill / arm pile / validate</t>
@@ -7081,7 +7231,7 @@
           <t>Manage subtab; target selected in inspector</t>
         </is>
       </c>
-      <c r="G106" s="29" t="inlineStr"/>
+      <c r="G106" s="29" t="n"/>
       <c r="H106" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_tools/input.rs</t>
@@ -7109,7 +7259,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="D107" s="29" t="inlineStr"/>
+      <c r="D107" s="29" t="n"/>
       <c r="E107" s="29" t="inlineStr">
         <is>
           <t>New detached inventory</t>
@@ -7120,13 +7270,13 @@
           <t>Items tab → Inventory Harness subtab</t>
         </is>
       </c>
-      <c r="G107" s="29" t="inlineStr"/>
+      <c r="G107" s="29" t="n"/>
       <c r="H107" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_harness.rs</t>
         </is>
       </c>
-      <c r="I107" s="29" t="inlineStr"/>
+      <c r="I107" s="29" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="29" t="inlineStr">
@@ -7144,7 +7294,7 @@
           <t>Del / Backspace</t>
         </is>
       </c>
-      <c r="D108" s="29" t="inlineStr"/>
+      <c r="D108" s="29" t="n"/>
       <c r="E108" s="29" t="inlineStr">
         <is>
           <t>Delete harness inventory</t>
@@ -7155,15 +7305,15 @@
           <t>Harness inventory active</t>
         </is>
       </c>
-      <c r="G108" s="29" t="inlineStr"/>
+      <c r="G108" s="29" t="n"/>
       <c r="H108" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_harness.rs</t>
         </is>
       </c>
-      <c r="I108" s="29" t="inlineStr"/>
-    </row>
-    <row r="109">
+      <c r="I108" s="29" t="n"/>
+    </row>
+    <row r="109" ht="30" customHeight="1" s="41">
       <c r="A109" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -7179,7 +7329,7 @@
           <t>A / U / O / V / H / M</t>
         </is>
       </c>
-      <c r="D109" s="29" t="inlineStr"/>
+      <c r="D109" s="29" t="n"/>
       <c r="E109" s="29" t="inlineStr">
         <is>
           <t>Add stack / unique / auto-sort / validate / split half / merge</t>
@@ -7190,13 +7340,13 @@
           <t>Harness inventory active</t>
         </is>
       </c>
-      <c r="G109" s="29" t="inlineStr"/>
+      <c r="G109" s="29" t="n"/>
       <c r="H109" s="29" t="inlineStr">
         <is>
           <t>src/dev/inventory_harness.rs</t>
         </is>
       </c>
-      <c r="I109" s="29" t="inlineStr"/>
+      <c r="I109" s="29" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="29" t="inlineStr">
@@ -7214,7 +7364,7 @@
           <t>V</t>
         </is>
       </c>
-      <c r="D110" s="29" t="inlineStr"/>
+      <c r="D110" s="29" t="n"/>
       <c r="E110" s="29" t="inlineStr">
         <is>
           <t>Validate world inventory</t>
@@ -7225,15 +7375,15 @@
           <t>World Tools tab</t>
         </is>
       </c>
-      <c r="G110" s="29" t="inlineStr"/>
+      <c r="G110" s="29" t="n"/>
       <c r="H110" s="29" t="inlineStr">
         <is>
           <t>src/dev/pile_harness.rs</t>
         </is>
       </c>
-      <c r="I110" s="29" t="inlineStr"/>
-    </row>
-    <row r="111">
+      <c r="I110" s="29" t="n"/>
+    </row>
+    <row r="111" ht="30" customHeight="1" s="41">
       <c r="A111" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -7249,7 +7399,7 @@
           <t>P / D / O / H / G / L</t>
         </is>
       </c>
-      <c r="D111" s="29" t="inlineStr"/>
+      <c r="D111" s="29" t="n"/>
       <c r="E111" s="29" t="inlineStr">
         <is>
           <t>Spawn pile / drop entry / drop one / half / pickup / loot</t>
@@ -7260,15 +7410,15 @@
           <t>World Tools; unit selected</t>
         </is>
       </c>
-      <c r="G111" s="29" t="inlineStr"/>
+      <c r="G111" s="29" t="n"/>
       <c r="H111" s="29" t="inlineStr">
         <is>
           <t>src/dev/pile_harness.rs</t>
         </is>
       </c>
-      <c r="I111" s="29" t="inlineStr"/>
-    </row>
-    <row r="112">
+      <c r="I111" s="29" t="n"/>
+    </row>
+    <row r="112" ht="30" customHeight="1" s="41">
       <c r="A112" s="29" t="inlineStr">
         <is>
           <t>Dev Mode</t>
@@ -7284,7 +7434,7 @@
           <t>J / B / C / Y / E</t>
         </is>
       </c>
-      <c r="D112" s="29" t="inlineStr"/>
+      <c r="D112" s="29" t="n"/>
       <c r="E112" s="29" t="inlineStr">
         <is>
           <t>Transaction log / wealth audit / create treasury / inspect / deposit</t>
@@ -7295,13 +7445,13 @@
           <t>World Tools; building selected (except J/B)</t>
         </is>
       </c>
-      <c r="G112" s="29" t="inlineStr"/>
+      <c r="G112" s="29" t="n"/>
       <c r="H112" s="29" t="inlineStr">
         <is>
           <t>src/dev/treasury_harness.rs</t>
         </is>
       </c>
-      <c r="I112" s="29" t="inlineStr"/>
+      <c r="I112" s="29" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:I112"/>
@@ -7318,13 +7468,13 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7.42578125" bestFit="1" customWidth="1" style="38" min="1" max="1"/>
-    <col width="45.140625" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
-    <col width="10.85546875" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
-    <col width="12.28515625" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" style="38" min="6" max="6"/>
-    <col width="33.28515625" bestFit="1" customWidth="1" style="38" min="7" max="7"/>
+    <col width="7.42578125" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
+    <col width="45.140625" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="41" min="3" max="3"/>
+    <col width="10.85546875" bestFit="1" customWidth="1" style="41" min="4" max="4"/>
+    <col width="12.28515625" bestFit="1" customWidth="1" style="41" min="5" max="5"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="41" min="6" max="6"/>
+    <col width="33.28515625" bestFit="1" customWidth="1" style="41" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7484,9 +7634,9 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22.85546875" customWidth="1" style="38" min="1" max="1"/>
-    <col width="19" customWidth="1" style="38" min="2" max="2"/>
-    <col width="38.140625" customWidth="1" style="38" min="3" max="4"/>
+    <col width="22.85546875" customWidth="1" style="41" min="1" max="1"/>
+    <col width="19" customWidth="1" style="41" min="2" max="2"/>
+    <col width="38.140625" customWidth="1" style="41" min="3" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7533,8 +7683,8 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18.75" customHeight="1" s="38">
-      <c r="A9" s="39" t="n"/>
+    <row r="9" ht="18.75" customHeight="1" s="41">
+      <c r="A9" s="42" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n"/>
@@ -7560,21 +7710,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:Y33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7.140625" bestFit="1" customWidth="1" style="38" min="1" max="1"/>
-    <col width="14.42578125" customWidth="1" style="38" min="2" max="2"/>
-    <col width="7.5703125" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
-    <col width="24.140625" customWidth="1" style="38" min="4" max="4"/>
-    <col width="5.85546875" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
-    <col width="8.28515625" bestFit="1" customWidth="1" style="38" min="6" max="6"/>
-    <col width="8.7109375" bestFit="1" customWidth="1" style="38" min="7" max="7"/>
-    <col width="9.42578125" bestFit="1" customWidth="1" style="38" min="8" max="8"/>
-    <col width="12.42578125" bestFit="1" customWidth="1" style="38" min="9" max="9"/>
-    <col width="6.5703125" bestFit="1" customWidth="1" style="38" min="10" max="10"/>
-    <col width="9.5703125" bestFit="1" customWidth="1" style="38" min="11" max="11"/>
-    <col width="11.7109375" bestFit="1" customWidth="1" style="38" min="12" max="12"/>
+    <col width="7.140625" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
+    <col width="14.42578125" customWidth="1" style="41" min="2" max="2"/>
+    <col width="7.5703125" bestFit="1" customWidth="1" style="41" min="3" max="3"/>
+    <col width="24.140625" customWidth="1" style="41" min="4" max="4"/>
+    <col width="5.85546875" bestFit="1" customWidth="1" style="41" min="5" max="5"/>
+    <col width="8.28515625" bestFit="1" customWidth="1" style="41" min="6" max="6"/>
+    <col width="8.7109375" bestFit="1" customWidth="1" style="41" min="7" max="7"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" style="41" min="8" max="8"/>
+    <col width="12.42578125" bestFit="1" customWidth="1" style="41" min="9" max="9"/>
+    <col width="6.5703125" bestFit="1" customWidth="1" style="41" min="10" max="10"/>
+    <col width="9.5703125" bestFit="1" customWidth="1" style="41" min="11" max="11"/>
+    <col width="11.7109375" bestFit="1" customWidth="1" style="41" min="12" max="12"/>
+    <col width="17.85546875" customWidth="1" style="41" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7678,6 +7829,31 @@
           <t>Enabled</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Default Weapon ID</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Rotation Correction X Deg</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Rotation Correction Y Deg</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Rotation Correction Z Deg</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Turn Speed Deg/s</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -7748,6 +7924,17 @@
         <is>
           <t>Y</t>
         </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>weapon_fists</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>90</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>540</v>
       </c>
     </row>
     <row r="3">
@@ -7826,9 +8013,101 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>weapon_claws</t>
+        </is>
+      </c>
+      <c r="Y3" t="n">
+        <v>720</v>
+      </c>
     </row>
     <row r="4">
-      <c r="O4" s="11" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>U-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cavecrawler</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Wild</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>assets\units\cavecrawler.glb</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>45</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>31</v>
+      </c>
+      <c r="N4" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="O4" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>45</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>cavecrawler</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>weapon_cavecrawler_claws</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>180</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="5">
       <c r="O5" s="11" t="n"/>
@@ -7910,7 +8189,8 @@
       <c r="N26" s="10" t="n"/>
       <c r="O26" s="12" t="n"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1" s="38">
+    <row r="27"/>
+    <row r="28" ht="15.75" customHeight="1" s="41">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>UNIT STATISTICS</t>
@@ -8025,38 +8305,38 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="98.28515625" customWidth="1" style="29" min="1" max="1"/>
-    <col width="12.5703125" customWidth="1" style="38" min="2" max="2"/>
+    <col width="12.5703125" customWidth="1" style="41" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="38">
+    <row r="1" ht="18" customHeight="1" s="41">
       <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Chasma — Setting Summary</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="75" customHeight="1" s="38">
+    <row r="3" ht="75" customHeight="1" s="41">
       <c r="A3" s="29" t="inlineStr">
         <is>
           <t>Humanity arrived on an inhabited alien world aboard a massive colony ship. During descent, the vessel catastrophically broke apart. The crew compartments scattered across the planet, while the main body of the ship—containing the majority of humanity's advanced technology—crashed near the center of the world. The survivors lacked the manpower and resources to reclaim it, and over generations humanity fell into fragmented settlements, preserving only pieces of their former knowledge.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1" s="38">
+    <row r="4" ht="45" customHeight="1" s="41">
       <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Today, the wreck remains the most valuable location on the planet. Every major civilization has a different vision for its future, creating a world of uneasy alliances, trade, proxy wars, and territorial conflict.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="38">
+    <row r="6" ht="18" customHeight="1" s="41">
       <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Humans</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1" s="38">
+    <row r="8" ht="45" customHeight="1" s="41">
       <c r="A8" s="29" t="inlineStr">
         <is>
           <t>The most intelligent and adaptable race, but also the most fractured. Their greatest strength is their potential to recover and understand lost technology. Human factions compete among themselves over how the old world should be rebuilt.</t>
@@ -8070,14 +8350,14 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="38">
+    <row r="11" ht="18" customHeight="1" s="41">
       <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Y'aratan</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1" s="38">
+    <row r="13" ht="60" customHeight="1" s="41">
       <c r="A13" s="29" t="inlineStr">
         <is>
           <t>An insectoid civilization roughly equivalent to medieval humans in technology. Originally organized around rigid biological castes and queens, increasing intelligence is causing individuals to question their assigned roles. Some queens seek to embrace human technology and evolve beyond their origins, while others view it as a corruption of the hive.</t>
@@ -8091,14 +8371,14 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="38">
+    <row r="16" ht="18" customHeight="1" s="41">
       <c r="A16" s="30" t="inlineStr">
         <is>
           <t>Gra-Gu</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1" s="38">
+    <row r="18" ht="60" customHeight="1" s="41">
       <c r="A18" s="29" t="inlineStr">
         <is>
           <t>Silicon-based beings living primarily in the mountains. Slow-moving, immensely durable, and operating on a vastly different perception of time, they are territorial but rarely aggressive. They witnessed humanity's technological power shortly after the crash and were deeply disturbed by what they saw. To them, the wreck is not a treasure—it is a danger.</t>
@@ -8112,14 +8392,14 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1" s="38">
+    <row r="21" ht="18" customHeight="1" s="41">
       <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Rhal</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1" s="38">
+    <row r="23" ht="60" customHeight="1" s="41">
       <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Digitigrade mammalian nomads known for their speed, endurance, and mastery of logistics. They maintain the trade routes connecting distant civilizations and are generally trusted more than any government or faction. While they rarely wage war, they understand better than anyone how valuable the crashed ship could become.</t>
@@ -8133,7 +8413,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1" s="38">
+    <row r="26" ht="18" customHeight="1" s="41">
       <c r="A26" s="30" t="inlineStr">
         <is>
           <t>Major Conflicts</t>
@@ -8234,7 +8514,7 @@
   <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="38" thickBot="1">
+    <row r="1" ht="15.75" customHeight="1" s="41" thickBot="1">
       <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Item ID</t>
@@ -9425,13 +9705,13 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.42578125" customWidth="1" style="38" min="1" max="1"/>
-    <col width="17.85546875" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="39.42578125" customWidth="1" style="38" min="3" max="3"/>
-    <col width="18.28515625" customWidth="1" style="38" min="5" max="5"/>
-    <col width="17.28515625" bestFit="1" customWidth="1" style="38" min="6" max="7"/>
-    <col width="17.28515625" customWidth="1" style="38" min="8" max="8"/>
-    <col width="18.28515625" customWidth="1" style="38" min="9" max="9"/>
+    <col width="13.42578125" customWidth="1" style="41" min="1" max="1"/>
+    <col width="17.85546875" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="39.42578125" customWidth="1" style="41" min="3" max="3"/>
+    <col width="18.28515625" customWidth="1" style="41" min="5" max="5"/>
+    <col width="17.28515625" bestFit="1" customWidth="1" style="41" min="6" max="7"/>
+    <col width="17.28515625" customWidth="1" style="41" min="8" max="8"/>
+    <col width="18.28515625" customWidth="1" style="41" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10008,7 +10288,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" s="38">
+    <row r="14" ht="15.75" customHeight="1" s="41">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>FACTION RELATIONSHIPS</t>

</xml_diff>

<commit_message>
More item fixes and matching to excel importer
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -21,6 +21,7 @@
     <sheet name="Animation Profiles" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Building Categories" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Buildings" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Item Categories" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hotkeys'!$A$4:$I$112</definedName>
@@ -2632,7 +2633,6 @@
           <t>CrawlForward</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>3.5</v>
       </c>
@@ -2651,7 +2651,6 @@
           <t>GetHit1</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>CrawlLeft</t>
@@ -3189,6 +3188,247 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Sort Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Trade currency and coinage</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Raw Material</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Unprocessed resources</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Melee and ranged weapons</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ammo</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ammunition</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ammunition and bolts</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Armor</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Wearable protection</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Consumable</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Consumable supplies</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Edible goods</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>quest</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Quest</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Quest and story items</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -8189,7 +8429,6 @@
       <c r="N26" s="10" t="n"/>
       <c r="O26" s="12" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28" ht="15.75" customHeight="1" s="41">
       <c r="A28" s="7" t="inlineStr">
         <is>
@@ -8511,56 +8750,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="41" thickBot="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Item ID</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="17" t="inlineStr">
-        <is>
-          <t>Stack Size</t>
-        </is>
-      </c>
-      <c r="E1" s="17" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Width</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Stackable</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Max Stack</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Mass Grams</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Base Value</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="G1" s="17" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Rarity</t>
         </is>
       </c>
-      <c r="H1" s="17" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Craft Recipe</t>
         </is>
       </c>
-      <c r="I1" s="17" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="J1" s="18" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Value/Weight</t>
         </is>
@@ -8569,1124 +8828,1581 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>I-0001</t>
+          <t>gold</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>999</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Physical gold coins carried as stackable currency.</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>iron_ore</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Iron Ore</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
         <v>50</v>
       </c>
-      <c r="E2" t="n">
+      <c r="H3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Raw iron for smelting</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Raw iron for smelting</t>
-        </is>
-      </c>
-      <c r="J2">
+      <c r="N3">
         <f>IF(F2&gt;0,ROUND(E2/F2,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>I-0002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>copper_ore</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Copper Ore</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>50</v>
       </c>
-      <c r="E3" t="n">
+      <c r="H4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Raw copper for smelting</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
         <v>4</v>
       </c>
-      <c r="F3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Raw copper for smelting</t>
-        </is>
-      </c>
-      <c r="J3">
+      <c r="N4">
         <f>IF(F3&gt;0,ROUND(E3/F3,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>I-0003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>iron_bar</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Iron Bar</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>20</v>
       </c>
-      <c r="E4" t="n">
+      <c r="H5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Refined iron</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
         <v>15</v>
       </c>
-      <c r="F4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>2x Iron Ore</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Refined iron</t>
-        </is>
-      </c>
-      <c r="J4">
+      <c r="N5">
         <f>IF(F4&gt;0,ROUND(E4/F4,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>I-0004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>copper_bar</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Copper Bar</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
         <v>20</v>
       </c>
-      <c r="E5" t="n">
+      <c r="H6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Refined copper</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
         <v>12</v>
       </c>
-      <c r="F5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>2x Copper Ore</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Refined copper</t>
-        </is>
-      </c>
-      <c r="J5">
+      <c r="N6">
         <f>IF(F5&gt;0,ROUND(E5/F5,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>I-0005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>scrap_metal</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Scrap Metal</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
         <v>30</v>
       </c>
-      <c r="E6" t="n">
+      <c r="H7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Salvaged metal</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
         <v>3</v>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Salvaged metal</t>
-        </is>
-      </c>
-      <c r="J6">
+      <c r="N7">
         <f>IF(F6&gt;0,ROUND(E6/F6,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>I-0006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ancient_parts</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Ancient Parts</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
         <v>10</v>
       </c>
-      <c r="E7" t="n">
+      <c r="H8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Pre-war technology</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
         <v>100</v>
       </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Pre-war technology</t>
-        </is>
-      </c>
-      <c r="J7">
+      <c r="N8">
         <f>IF(F7&gt;0,ROUND(E7/F7,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>I-0007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>electronics</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
         <v>15</v>
       </c>
-      <c r="E8" t="n">
+      <c r="H9" t="n">
+        <v>500</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Circuits and wires</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
         <v>50</v>
       </c>
-      <c r="F8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Uncommon</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Circuits and wires</t>
-        </is>
-      </c>
-      <c r="J8">
+      <c r="N9">
         <f>IF(F8&gt;0,ROUND(E8/F8,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>I-0008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>wood</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
         <v>50</v>
       </c>
-      <c r="E9" t="n">
+      <c r="H10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Building material</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
         <v>2</v>
       </c>
-      <c r="F9" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Building material</t>
-        </is>
-      </c>
-      <c r="J9">
+      <c r="N10">
         <f>IF(F9&gt;0,ROUND(E9/F9,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>I-0009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stone</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
         <v>50</v>
       </c>
-      <c r="E10" t="n">
+      <c r="H11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Building material</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Building material</t>
-        </is>
-      </c>
-      <c r="J10">
+      <c r="N11">
         <f>IF(F10&gt;0,ROUND(E10/F10,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>I-0010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>plant_fiber</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Plant Fiber</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>raw_material</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
         <v>50</v>
       </c>
-      <c r="E11" t="n">
+      <c r="H12" t="n">
+        <v>200</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>For bandages and rope</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>For bandages and rope</t>
-        </is>
-      </c>
-      <c r="J11">
+      <c r="N12">
         <f>IF(F11&gt;0,ROUND(E11/F11,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>I-0011</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>rusty_sword</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Rusty Sword</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
         <v>1</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Basic melee weapon</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
         <v>50</v>
       </c>
-      <c r="F12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Basic melee weapon</t>
-        </is>
-      </c>
-      <c r="J12">
+      <c r="N13">
         <f>IF(F12&gt;0,ROUND(E12/F12,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>I-0012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>iron_sword</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Iron Sword</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Reliable blade</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
         <v>150</v>
       </c>
-      <c r="F13" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Uncommon</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>5x Iron Bar</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Reliable blade</t>
-        </is>
-      </c>
-      <c r="J13">
+      <c r="N14">
         <f>IF(F13&gt;0,ROUND(E13/F13,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>I-0013</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>machete</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Machete</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>1</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Fast slashing weapon</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
         <v>80</v>
       </c>
-      <c r="F14" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>3x Iron Bar</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Fast slashing weapon</t>
-        </is>
-      </c>
-      <c r="J14">
+      <c r="N15">
         <f>IF(F14&gt;0,ROUND(E14/F14,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>I-0014</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sledgehammer</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Sledgehammer</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="n">
+      <c r="H16" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Heavy blunt weapon</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
         <v>120</v>
       </c>
-      <c r="F15" t="n">
-        <v>8</v>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Uncommon</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>4x Iron Bar, 2x Wood</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Heavy blunt weapon</t>
-        </is>
-      </c>
-      <c r="J15">
+      <c r="N16">
         <f>IF(F15&gt;0,ROUND(E15/F15,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>I-0015</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>crossbow</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Crossbow</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Weapon</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
         <v>1</v>
       </c>
-      <c r="E16" t="n">
+      <c r="H17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Ranged weapon</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
         <v>200</v>
       </c>
-      <c r="F16" t="n">
-        <v>5</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Uncommon</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>3x Iron Bar, 4x Wood</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Ranged weapon</t>
-        </is>
-      </c>
-      <c r="J16">
+      <c r="N17">
         <f>IF(F16&gt;0,ROUND(E16/F16,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>I-0016</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>bolt</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Bolt</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Ammo</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ammo</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
         <v>50</v>
       </c>
-      <c r="E17" t="n">
+      <c r="H18" t="n">
+        <v>100</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Crossbow ammo</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
         <v>2</v>
       </c>
-      <c r="F17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>1x Iron Bar = 10</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Crossbow ammo</t>
-        </is>
-      </c>
-      <c r="J17">
+      <c r="N18">
         <f>IF(F17&gt;0,ROUND(E17/F17,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>I-0017</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ragged_clothes</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Ragged Clothes</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Armor</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
         <v>1</v>
       </c>
-      <c r="E18" t="n">
+      <c r="H19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Barely protection</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
         <v>10</v>
       </c>
-      <c r="F18" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Barely protection</t>
-        </is>
-      </c>
-      <c r="J18">
+      <c r="N19">
         <f>IF(F18&gt;0,ROUND(E18/F18,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>I-0018</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>leather_armor</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Leather Armor</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Armor</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="E19" t="n">
+      <c r="H20" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Light protection</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
         <v>100</v>
       </c>
-      <c r="F19" t="n">
-        <v>6</v>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>5x Leather</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Light protection</t>
-        </is>
-      </c>
-      <c r="J19">
+      <c r="N20">
         <f>IF(F19&gt;0,ROUND(E19/F19,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>I-0019</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>iron_plate_armor</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Iron Plate Armor</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Armor</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="n">
+      <c r="H21" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Heavy protection</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
         <v>300</v>
       </c>
-      <c r="F20" t="n">
-        <v>15</v>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Uncommon</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>10x Iron Bar</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Heavy protection</t>
-        </is>
-      </c>
-      <c r="J20">
+      <c r="N21">
         <f>IF(F20&gt;0,ROUND(E20/F20,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>I-0020</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>bandage</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Bandage</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
         <v>20</v>
       </c>
-      <c r="E21" t="n">
+      <c r="H22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Heals 10 HP</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
         <v>5</v>
       </c>
-      <c r="F21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>2x Plant Fiber</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Heals 10 HP</t>
-        </is>
-      </c>
-      <c r="J21">
+      <c r="N22">
         <f>IF(F21&gt;0,ROUND(E21/F21,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>I-0021</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>med_kit</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Med Kit</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
         <v>10</v>
       </c>
-      <c r="E22" t="n">
+      <c r="H23" t="n">
+        <v>500</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Heals 50 HP</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
         <v>50</v>
       </c>
-      <c r="F22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>Uncommon</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>5x Bandage, Alcohol</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Heals 50 HP</t>
-        </is>
-      </c>
-      <c r="J22">
+      <c r="N23">
         <f>IF(F22&gt;0,ROUND(E22/F22,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>I-0022</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>dried_meat</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Dried Meat</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
         <v>20</v>
       </c>
-      <c r="E23" t="n">
+      <c r="H24" t="n">
+        <v>300</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Restores 20 hunger</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
         <v>8</v>
       </c>
-      <c r="F23" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>1x Raw Meat</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Restores 20 hunger</t>
-        </is>
-      </c>
-      <c r="J23">
+      <c r="N24">
         <f>IF(F23&gt;0,ROUND(E23/F23,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>I-0023</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cactus_flesh</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>Cactus Flesh</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
         <v>20</v>
       </c>
-      <c r="E24" t="n">
+      <c r="H25" t="n">
+        <v>200</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Restores 10 hunger</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
         <v>3</v>
       </c>
-      <c r="F24" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Restores 10 hunger</t>
-        </is>
-      </c>
-      <c r="J24">
+      <c r="N25">
         <f>IF(F24&gt;0,ROUND(E24/F24,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>I-0024</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>water_flask</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Water Flask</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
         <v>5</v>
       </c>
-      <c r="E25" t="n">
+      <c r="H26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Holds water</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
         <v>15</v>
       </c>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>2x Leather</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Holds water</t>
-        </is>
-      </c>
-      <c r="J25">
+      <c r="N26">
         <f>IF(F25&gt;0,ROUND(E25/F25,1),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>I-0025</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>data_chip</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Data Chip</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>Quest</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="n">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>quest</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
         <v>5</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="H27" t="n">
+        <v>100</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Contains ancient data</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
         <v>500</v>
       </c>
-      <c r="F26" s="10" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>Rare</t>
         </is>
       </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>Contains ancient data</t>
-        </is>
-      </c>
-      <c r="J26" s="10">
+      <c r="N27">
         <f>IF(F26&gt;0,ROUND(E26/F26,1),"-")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Reputation and debug overlay addition
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -22,6 +22,9 @@
     <sheet name="Building Categories" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Buildings" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Item Categories" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Species" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Rel Faction Faction" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Rel Faction Species" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hotkeys'!$A$4:$I$112</definedName>
@@ -504,14 +507,9 @@
         <t>STORED — design metadata only; not runtime ownership</t>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>USED — GLB path → render key (e.g. robot); blank = no mesh</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>STORED — catalog stat; no gameplay effect yet</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -536,12 +534,12 @@
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>STORED — catalog stat only; does NOT affect move speed (use Move Speed)</t>
+        <t>STORED — catalog stat; no gameplay effect yet</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>STORED — catalog stat; no gameplay effect yet</t>
+        <t>STORED — catalog stat only; does NOT affect move speed (use Move Speed)</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -551,35 +549,40 @@
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>IGNORED — sheet formula only; importer skips this column</t>
+        <t>STORED — catalog stat; no gameplay effect yet</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>STORED — imported float; no gameplay effect yet (script writes computed value)</t>
+        <t>IGNORED — sheet formula only; importer skips this column</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>USED — required string (Elite/Veteran/…); imported to catalog (script writes computed value)</t>
+        <t>STORED — imported float; no gameplay effect yet (script writes computed value)</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>USED — meters/sec for movement simulation (authoritative for speed)</t>
+        <t>USED — required string (Elite/Veteran/…); imported to catalog (script writes computed value)</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>USED — meters; selection ring + steering radius</t>
+        <t>USED — meters/sec for movement simulation (authoritative for speed)</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
+        <t>USED — meters; selection ring + steering radius</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
         <t>USED — degrees; max walkable terrain slope for pathfinding</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t>USED — Y/N; N excludes row from imported catalog</t>
       </text>
@@ -3429,6 +3432,302 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Species Key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>robot</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Robot</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Player humanoid construct</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fox</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fox</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Small canid companion</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cavecrawler</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cavecrawler</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Subterranean predator</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Faction -&gt; Faction</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>bandits</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>raiders</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>nomads</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>town</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>slavers</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tech_hunters</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>scavs</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dominion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-300</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>bandits</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>raiders</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nomads</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>town</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>slavers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tech_hunters</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>scavs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dominion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Faction -&gt; Species</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>robot</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fox</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cavecrawler</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7950,7 +8249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y33"/>
+  <dimension ref="A1:AA33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.140625" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
@@ -7981,117 +8280,127 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Faction</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
+          <t>Faction Key</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Species Key</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>File Path</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Base HP</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Dexterity</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Constitution</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Agility</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Charisma</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Intelligence</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>Total Stats</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>Power Rating</t>
         </is>
       </c>
-      <c r="O1" s="9" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="P1" s="36" t="inlineStr">
+      <c r="Q1" s="36" t="inlineStr">
         <is>
           <t>Move Speed</t>
         </is>
       </c>
-      <c r="Q1" s="36" t="inlineStr">
+      <c r="R1" s="36" t="inlineStr">
         <is>
           <t>Collision Radius</t>
         </is>
       </c>
-      <c r="R1" s="36" t="inlineStr">
+      <c r="S1" s="36" t="inlineStr">
         <is>
           <t>Max Slope</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Animation Profile</t>
         </is>
       </c>
-      <c r="T1" s="36" t="inlineStr">
+      <c r="U1" s="36" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Default Weapon ID</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Rotation Correction X Deg</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Rotation Correction Y Deg</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Rotation Correction Z Deg</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Turn Speed Deg/s</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Sight Range</t>
         </is>
       </c>
     </row>
@@ -8108,73 +8417,81 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>robot</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>assets\units\robot.glb</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="F2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="H2" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="I2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="J2" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="K2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="L2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="L2" s="1" t="n">
+      <c r="M2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>48</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>65.40000000000001</v>
       </c>
-      <c r="O2" s="11" t="inlineStr">
+      <c r="P2" s="11" t="inlineStr">
         <is>
           <t>Elite</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>9</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>0.68</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>40</v>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>weapon_fists</t>
         </is>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>90</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>540</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -8190,76 +8507,84 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>fox</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>assets\units\fox.glb</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>25</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>4</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>12</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>6</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>15</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>8</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>7</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <f>SUM(G3:L3)</f>
         <v/>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>70</v>
       </c>
-      <c r="O3" s="11" t="inlineStr">
+      <c r="P3" s="11" t="inlineStr">
         <is>
           <t>Creep</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>14</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>1.25</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>50</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>fox</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>weapon_claws</t>
         </is>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>720</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -8275,148 +8600,155 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wild</t>
+          <t>wild</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>cavecrawler</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>assets\units\cavecrawler.glb</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>45</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>6</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>7</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>5</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>2</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>3</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>31</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>53.3</v>
       </c>
-      <c r="O4" s="11" t="inlineStr">
+      <c r="P4" s="11" t="inlineStr">
         <is>
           <t>Elite</t>
         </is>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>3.5</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>1.1</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>45</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>cavecrawler</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>weapon_cavecrawler_claws</t>
         </is>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>180</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>360</v>
       </c>
+      <c r="AA4" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="5">
-      <c r="O5" s="11" t="n"/>
+      <c r="P5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="O6" s="11" t="n"/>
+      <c r="P6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="O8" s="11" t="n"/>
+      <c r="P8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="O10" s="11" t="n"/>
+      <c r="P10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="O11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="O12" s="11" t="n"/>
+      <c r="P12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="O13" s="11" t="n"/>
+      <c r="P13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="O14" s="11" t="n"/>
+      <c r="P14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="O15" s="11" t="n"/>
+      <c r="P15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="O16" s="11" t="n"/>
+      <c r="P16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="O20" s="11" t="n"/>
+      <c r="P20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="O22" s="11" t="n"/>
+      <c r="P22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="O23" s="11" t="n"/>
+      <c r="P23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="O24" s="11" t="n"/>
+      <c r="P24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="O25" s="11" t="n"/>
+      <c r="P25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="10" t="n"/>
       <c r="G26" s="10" t="n"/>
@@ -8427,13 +8759,17 @@
       <c r="L26" s="10" t="n"/>
       <c r="M26" s="10" t="n"/>
       <c r="N26" s="10" t="n"/>
-      <c r="O26" s="12" t="n"/>
+      <c r="O26" s="10" t="n"/>
+      <c r="P26" s="12" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="41">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>UNIT STATISTICS</t>
         </is>
+      </c>
+      <c r="AA28" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="29">
@@ -8446,14 +8782,27 @@
         <f>COUNTA(A2:A26)</f>
         <v/>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>counta_a2_a26</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Elite Units:</t>
         </is>
       </c>
-      <c r="F29" s="28">
+      <c r="G29" s="28">
         <f>COUNTIF(O2:O26,"Elite")</f>
         <v/>
+      </c>
+      <c r="AA29" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="30">
@@ -8466,14 +8815,27 @@
         <f>ROUND(AVERAGE(N2:N26),1)</f>
         <v/>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>round_average_n2_n26_1</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Veteran Units:</t>
         </is>
       </c>
-      <c r="F30" s="28">
+      <c r="G30" s="28">
         <f>COUNTIF(O2:O26,"Veteran")</f>
         <v/>
+      </c>
+      <c r="AA30" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="31">
@@ -8486,14 +8848,27 @@
         <f>INDEX(B2:B26,MATCH(MAX(N2:N26),N2:N26,0))</f>
         <v/>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>index_b2_b26_match_max_n2_n26_n2_n26_0</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Regular Units:</t>
         </is>
       </c>
-      <c r="F31" s="28">
+      <c r="G31" s="28">
         <f>COUNTIF(O2:O26,"Regular")</f>
         <v/>
+      </c>
+      <c r="AA31" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="32">
@@ -8506,14 +8881,27 @@
         <f>COUNTIF(C2:C26,"Wild")</f>
         <v/>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>countif_c2_c26_wild</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Rookie Units:</t>
         </is>
       </c>
-      <c r="F32" s="28">
+      <c r="G32" s="28">
         <f>COUNTIF(O2:O26,"Rookie")</f>
         <v/>
+      </c>
+      <c r="AA32" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="33">
@@ -8525,6 +8913,19 @@
       <c r="B33" s="27">
         <f>COUNTIF(C2:C26,"Bandits")</f>
         <v/>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>countif_c2_c26_bandits</t>
+        </is>
+      </c>
+      <c r="AA33" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -10539,25 +10940,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Faction Key</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Faction ID</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="20" t="inlineStr">
-        <is>
-          <t>Disposition</t>
-        </is>
-      </c>
       <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Territory</t>
@@ -10581,25 +10982,30 @@
       <c r="H1" s="20" t="inlineStr">
         <is>
           <t>Description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>F-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Variable</t>
@@ -10623,25 +11029,30 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>The player's faction</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>F-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Wild</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Wilderness</t>
@@ -10665,25 +11076,30 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>Wild creatures and beasts</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>bandits</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>F-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Bandits</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Roads, Ruins</t>
@@ -10707,25 +11123,30 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>Opportunistic raiders</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>raiders</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>F-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Raiders</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Badlands</t>
@@ -10749,25 +11170,30 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>Organized criminal group</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>nomads</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>F-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Nomads</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Desert</t>
@@ -10791,25 +11217,30 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>Wandering traders</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>town</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>F-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Town</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Friendly</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Settlements</t>
@@ -10833,25 +11264,30 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>Civilization survivors</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>slavers</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>F-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Slavers</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>Slave camps</t>
@@ -10875,25 +11311,30 @@
       <c r="H8" t="inlineStr">
         <is>
           <t>Human traffickers</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>tech_hunters</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>F-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Tech Hunters</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Ruins</t>
@@ -10917,25 +11358,30 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>Relic seekers</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>scavs</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>F-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Scavs</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Everywhere</t>
@@ -10961,23 +11407,28 @@
           <t>Scrap collectors</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dominion</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>F-0010</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>The Dominion</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
           <t>East Chasma</t>
@@ -11003,206 +11454,13 @@
           <t>Authoritarian empire</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="15.75" customHeight="1" s="41">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>FACTION RELATIONSHIPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>From \ To</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>Bandits</t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>Nomads</t>
-        </is>
-      </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Town</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>Slavers</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="inlineStr">
-        <is>
-          <t>Tech Hunters</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>Bandits</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>Nomads</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Friendly</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="21" t="inlineStr">
-        <is>
-          <t>Town</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Friendly</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Friendly</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>Slavers</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>Tech Hunters</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Hostile</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Friendly</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1" s="41"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>